<commit_message>
Add Posto Gangorra licence RLO-0422 with folder-57 documents; update spreadsheet
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QfG4bt12JG3GE3pGHANk8N
</commit_message>
<xml_diff>
--- a/pendencias-condicionantes-2026-10-23.xlsx
+++ b/pendencias-condicionantes-2026-10-23.xlsx
@@ -14,8 +14,8 @@
     <sheet name="Licenças que faltam" sheetId="4" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Pendências!$A$1:$R$145</definedName>
-    <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">'Por empresa'!$A$1:$F$50</definedName>
+    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">Pendências!$A$1:$R$149</definedName>
+    <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">'Por empresa'!$A$1:$F$51</definedName>
   </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1591" uniqueCount="350">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1632" uniqueCount="357">
   <si>
     <t xml:space="preserve">Condicionantes ambientais – pendências</t>
   </si>
@@ -818,6 +818,27 @@
     <t xml:space="preserve">Documento na pasta: AVCB emitido em 15/04/2025</t>
   </si>
   <si>
+    <t xml:space="preserve">Posto Gangorra Ltda</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rafael Fernandes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">03.365.159/0001-06</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2020-150998/TEC/RLO-0422</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Licença vale até 04/08/2026 (pedido ≥120 dias antes)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Documento na pasta: Coleta em 15/06/2026 (pasta 57, CNPJ 19.688.384/0001-05: confirmar se é a mesma empresa) → +3 meses</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Documento na pasta: Verificação de 14/11/2025 (pasta 57); renovação anual</t>
+  </si>
+  <si>
     <t xml:space="preserve">Posto Ln Ltda</t>
   </si>
   <si>
@@ -1043,13 +1064,13 @@
     <t xml:space="preserve">Pasta 55 só tem ANP; falta a licença</t>
   </si>
   <si>
-    <t xml:space="preserve">Alexandre's Combustíveis (Posto Gangorra)</t>
+    <t xml:space="preserve">Alexandre's Combustíveis (pasta 57)</t>
   </si>
   <si>
     <t xml:space="preserve">19.688.384/0001-05</t>
   </si>
   <si>
-    <t xml:space="preserve">Pasta 57 tem TOG, ANP, INMETRO e laudo; falta a licença</t>
+    <t xml:space="preserve">Os documentos da pasta 57 foram associados à licença do Posto Gangorra (CNPJ 03.365.159/0001-06). Confirmar se são a mesma empresa e, se não, enviar a licença do Alexandre's</t>
   </si>
   <si>
     <t xml:space="preserve">Gildo Alves de Carvalho (Posto Boa Vista)</t>
@@ -1785,20 +1806,20 @@
         <v>9</v>
       </c>
       <c r="B6" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$H$2:$H$145,$A6,Pendências!$J$2:$J$145,"Vencida")</f>
-        <v>12</v>
+        <f aca="false">COUNTIFS(Pendências!$H$2:$H$149,$A6,Pendências!$J$2:$J$149,"Vencida")</f>
+        <v>13</v>
       </c>
       <c r="C6" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$H$2:$H$145,$A6,Pendências!$J$2:$J$145,"Sem data")</f>
+        <f aca="false">COUNTIFS(Pendências!$H$2:$H$149,$A6,Pendências!$J$2:$J$149,"Sem data")</f>
         <v>0</v>
       </c>
       <c r="D6" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$H$2:$H$145,$A6,Pendências!$J$2:$J$145,"Vence em breve")</f>
+        <f aca="false">COUNTIFS(Pendências!$H$2:$H$149,$A6,Pendências!$J$2:$J$149,"Vence em breve")</f>
         <v>0</v>
       </c>
       <c r="E6" s="7" t="n">
         <f aca="false">SUM(B6:D6)</f>
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1806,15 +1827,15 @@
         <v>10</v>
       </c>
       <c r="B7" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$H$2:$H$145,$A7,Pendências!$J$2:$J$145,"Vencida")</f>
+        <f aca="false">COUNTIFS(Pendências!$H$2:$H$149,$A7,Pendências!$J$2:$J$149,"Vencida")</f>
         <v>8</v>
       </c>
       <c r="C7" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$H$2:$H$145,$A7,Pendências!$J$2:$J$145,"Sem data")</f>
+        <f aca="false">COUNTIFS(Pendências!$H$2:$H$149,$A7,Pendências!$J$2:$J$149,"Sem data")</f>
         <v>0</v>
       </c>
       <c r="D7" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$H$2:$H$145,$A7,Pendências!$J$2:$J$145,"Vence em breve")</f>
+        <f aca="false">COUNTIFS(Pendências!$H$2:$H$149,$A7,Pendências!$J$2:$J$149,"Vence em breve")</f>
         <v>4</v>
       </c>
       <c r="E7" s="7" t="n">
@@ -1827,15 +1848,15 @@
         <v>11</v>
       </c>
       <c r="B8" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$H$2:$H$145,$A8,Pendências!$J$2:$J$145,"Vencida")</f>
+        <f aca="false">COUNTIFS(Pendências!$H$2:$H$149,$A8,Pendências!$J$2:$J$149,"Vencida")</f>
         <v>7</v>
       </c>
       <c r="C8" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$H$2:$H$145,$A8,Pendências!$J$2:$J$145,"Sem data")</f>
+        <f aca="false">COUNTIFS(Pendências!$H$2:$H$149,$A8,Pendências!$J$2:$J$149,"Sem data")</f>
         <v>0</v>
       </c>
       <c r="D8" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$H$2:$H$145,$A8,Pendências!$J$2:$J$145,"Vence em breve")</f>
+        <f aca="false">COUNTIFS(Pendências!$H$2:$H$149,$A8,Pendências!$J$2:$J$149,"Vence em breve")</f>
         <v>0</v>
       </c>
       <c r="E8" s="7" t="n">
@@ -1848,15 +1869,15 @@
         <v>12</v>
       </c>
       <c r="B9" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$H$2:$H$145,$A9,Pendências!$J$2:$J$145,"Vencida")</f>
+        <f aca="false">COUNTIFS(Pendências!$H$2:$H$149,$A9,Pendências!$J$2:$J$149,"Vencida")</f>
         <v>5</v>
       </c>
       <c r="C9" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$H$2:$H$145,$A9,Pendências!$J$2:$J$145,"Sem data")</f>
+        <f aca="false">COUNTIFS(Pendências!$H$2:$H$149,$A9,Pendências!$J$2:$J$149,"Sem data")</f>
         <v>0</v>
       </c>
       <c r="D9" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$H$2:$H$145,$A9,Pendências!$J$2:$J$145,"Vence em breve")</f>
+        <f aca="false">COUNTIFS(Pendências!$H$2:$H$149,$A9,Pendências!$J$2:$J$149,"Vence em breve")</f>
         <v>1</v>
       </c>
       <c r="E9" s="7" t="n">
@@ -1869,15 +1890,15 @@
         <v>13</v>
       </c>
       <c r="B10" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$H$2:$H$145,$A10,Pendências!$J$2:$J$145,"Vencida")</f>
+        <f aca="false">COUNTIFS(Pendências!$H$2:$H$149,$A10,Pendências!$J$2:$J$149,"Vencida")</f>
         <v>2</v>
       </c>
       <c r="C10" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$H$2:$H$145,$A10,Pendências!$J$2:$J$145,"Sem data")</f>
+        <f aca="false">COUNTIFS(Pendências!$H$2:$H$149,$A10,Pendências!$J$2:$J$149,"Sem data")</f>
         <v>1</v>
       </c>
       <c r="D10" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$H$2:$H$145,$A10,Pendências!$J$2:$J$145,"Vence em breve")</f>
+        <f aca="false">COUNTIFS(Pendências!$H$2:$H$149,$A10,Pendências!$J$2:$J$149,"Vence em breve")</f>
         <v>0</v>
       </c>
       <c r="E10" s="7" t="n">
@@ -1890,20 +1911,20 @@
         <v>14</v>
       </c>
       <c r="B11" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$H$2:$H$145,$A11,Pendências!$J$2:$J$145,"Vencida")</f>
+        <f aca="false">COUNTIFS(Pendências!$H$2:$H$149,$A11,Pendências!$J$2:$J$149,"Vencida")</f>
         <v>24</v>
       </c>
       <c r="C11" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$H$2:$H$145,$A11,Pendências!$J$2:$J$145,"Sem data")</f>
-        <v>10</v>
+        <f aca="false">COUNTIFS(Pendências!$H$2:$H$149,$A11,Pendências!$J$2:$J$149,"Sem data")</f>
+        <v>11</v>
       </c>
       <c r="D11" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$H$2:$H$145,$A11,Pendências!$J$2:$J$145,"Vence em breve")</f>
+        <f aca="false">COUNTIFS(Pendências!$H$2:$H$149,$A11,Pendências!$J$2:$J$149,"Vence em breve")</f>
         <v>4</v>
       </c>
       <c r="E11" s="7" t="n">
         <f aca="false">SUM(B11:D11)</f>
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1911,20 +1932,20 @@
         <v>15</v>
       </c>
       <c r="B12" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$H$2:$H$145,$A12,Pendências!$J$2:$J$145,"Vencida")</f>
-        <v>38</v>
+        <f aca="false">COUNTIFS(Pendências!$H$2:$H$149,$A12,Pendências!$J$2:$J$149,"Vencida")</f>
+        <v>39</v>
       </c>
       <c r="C12" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$H$2:$H$145,$A12,Pendências!$J$2:$J$145,"Sem data")</f>
+        <f aca="false">COUNTIFS(Pendências!$H$2:$H$149,$A12,Pendências!$J$2:$J$149,"Sem data")</f>
         <v>9</v>
       </c>
       <c r="D12" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$H$2:$H$145,$A12,Pendências!$J$2:$J$145,"Vence em breve")</f>
+        <f aca="false">COUNTIFS(Pendências!$H$2:$H$149,$A12,Pendências!$J$2:$J$149,"Vence em breve")</f>
         <v>0</v>
       </c>
       <c r="E12" s="7" t="n">
         <f aca="false">SUM(B12:D12)</f>
-        <v>47</v>
+        <v>48</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1932,20 +1953,20 @@
         <v>16</v>
       </c>
       <c r="B13" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$H$2:$H$145,$A13,Pendências!$J$2:$J$145,"Vencida")</f>
+        <f aca="false">COUNTIFS(Pendências!$H$2:$H$149,$A13,Pendências!$J$2:$J$149,"Vencida")</f>
         <v>1</v>
       </c>
       <c r="C13" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$H$2:$H$145,$A13,Pendências!$J$2:$J$145,"Sem data")</f>
+        <f aca="false">COUNTIFS(Pendências!$H$2:$H$149,$A13,Pendências!$J$2:$J$149,"Sem data")</f>
         <v>4</v>
       </c>
       <c r="D13" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$H$2:$H$145,$A13,Pendências!$J$2:$J$145,"Vence em breve")</f>
-        <v>3</v>
+        <f aca="false">COUNTIFS(Pendências!$H$2:$H$149,$A13,Pendências!$J$2:$J$149,"Vence em breve")</f>
+        <v>4</v>
       </c>
       <c r="E13" s="7" t="n">
         <f aca="false">SUM(B13:D13)</f>
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1953,15 +1974,15 @@
         <v>17</v>
       </c>
       <c r="B14" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$H$2:$H$145,$A14,Pendências!$J$2:$J$145,"Vencida")</f>
+        <f aca="false">COUNTIFS(Pendências!$H$2:$H$149,$A14,Pendências!$J$2:$J$149,"Vencida")</f>
         <v>1</v>
       </c>
       <c r="C14" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$H$2:$H$145,$A14,Pendências!$J$2:$J$145,"Sem data")</f>
+        <f aca="false">COUNTIFS(Pendências!$H$2:$H$149,$A14,Pendências!$J$2:$J$149,"Sem data")</f>
         <v>3</v>
       </c>
       <c r="D14" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$H$2:$H$145,$A14,Pendências!$J$2:$J$145,"Vence em breve")</f>
+        <f aca="false">COUNTIFS(Pendências!$H$2:$H$149,$A14,Pendências!$J$2:$J$149,"Vence em breve")</f>
         <v>0</v>
       </c>
       <c r="E14" s="7" t="n">
@@ -1974,15 +1995,15 @@
         <v>18</v>
       </c>
       <c r="B15" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$H$2:$H$145,$A15,Pendências!$J$2:$J$145,"Vencida")</f>
+        <f aca="false">COUNTIFS(Pendências!$H$2:$H$149,$A15,Pendências!$J$2:$J$149,"Vencida")</f>
         <v>0</v>
       </c>
       <c r="C15" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$H$2:$H$145,$A15,Pendências!$J$2:$J$145,"Sem data")</f>
+        <f aca="false">COUNTIFS(Pendências!$H$2:$H$149,$A15,Pendências!$J$2:$J$149,"Sem data")</f>
         <v>4</v>
       </c>
       <c r="D15" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$H$2:$H$145,$A15,Pendências!$J$2:$J$145,"Vence em breve")</f>
+        <f aca="false">COUNTIFS(Pendências!$H$2:$H$149,$A15,Pendências!$J$2:$J$149,"Vence em breve")</f>
         <v>0</v>
       </c>
       <c r="E15" s="7" t="n">
@@ -1995,15 +2016,15 @@
         <v>19</v>
       </c>
       <c r="B16" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$H$2:$H$145,$A16,Pendências!$J$2:$J$145,"Vencida")</f>
+        <f aca="false">COUNTIFS(Pendências!$H$2:$H$149,$A16,Pendências!$J$2:$J$149,"Vencida")</f>
         <v>0</v>
       </c>
       <c r="C16" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$H$2:$H$145,$A16,Pendências!$J$2:$J$145,"Sem data")</f>
+        <f aca="false">COUNTIFS(Pendências!$H$2:$H$149,$A16,Pendências!$J$2:$J$149,"Sem data")</f>
         <v>3</v>
       </c>
       <c r="D16" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$H$2:$H$145,$A16,Pendências!$J$2:$J$145,"Vence em breve")</f>
+        <f aca="false">COUNTIFS(Pendências!$H$2:$H$149,$A16,Pendências!$J$2:$J$149,"Vence em breve")</f>
         <v>0</v>
       </c>
       <c r="E16" s="7" t="n">
@@ -2017,19 +2038,19 @@
       </c>
       <c r="B17" s="8" t="n">
         <f aca="false">SUM(B6:B16)</f>
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="C17" s="8" t="n">
         <f aca="false">SUM(C6:C16)</f>
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="D17" s="8" t="n">
         <f aca="false">SUM(D6:D16)</f>
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E17" s="8" t="n">
         <f aca="false">SUM(E6:E16)</f>
-        <v>144</v>
+        <v>148</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2042,8 +2063,8 @@
         <v>22</v>
       </c>
       <c r="B20" s="6" t="n">
-        <f aca="false">COUNTIF(Pendências!$P$2:$P$145,A20)</f>
-        <v>144</v>
+        <f aca="false">COUNTIF(Pendências!$P$2:$P$149,A20)</f>
+        <v>148</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2051,7 +2072,7 @@
         <v>23</v>
       </c>
       <c r="B21" s="6" t="n">
-        <f aca="false">COUNTIF(Pendências!$P$2:$P$145,A21)</f>
+        <f aca="false">COUNTIF(Pendências!$P$2:$P$149,A21)</f>
         <v>0</v>
       </c>
     </row>
@@ -2060,7 +2081,7 @@
         <v>24</v>
       </c>
       <c r="B22" s="6" t="n">
-        <f aca="false">COUNTIF(Pendências!$P$2:$P$145,A22)</f>
+        <f aca="false">COUNTIF(Pendências!$P$2:$P$149,A22)</f>
         <v>0</v>
       </c>
     </row>
@@ -2069,7 +2090,7 @@
         <v>25</v>
       </c>
       <c r="B23" s="6" t="n">
-        <f aca="false">COUNTIF(Pendências!$P$2:$P$145,A23)</f>
+        <f aca="false">COUNTIF(Pendências!$P$2:$P$149,A23)</f>
         <v>0</v>
       </c>
     </row>
@@ -2078,7 +2099,7 @@
         <v>26</v>
       </c>
       <c r="B24" s="6" t="n">
-        <f aca="false">COUNTIF(Pendências!$P$2:$P$145,A24)</f>
+        <f aca="false">COUNTIF(Pendências!$P$2:$P$149,A24)</f>
         <v>0</v>
       </c>
     </row>
@@ -2103,7 +2124,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:R145"/>
+  <dimension ref="A1:R149"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="5"/>
@@ -7729,23 +7750,23 @@
         <v>266</v>
       </c>
       <c r="G112" s="12" t="n">
-        <v>46043</v>
+        <v>46238</v>
       </c>
       <c r="H112" s="10" t="s">
         <v>9</v>
       </c>
       <c r="I112" s="10" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="J112" s="10" t="s">
         <v>56</v>
       </c>
       <c r="K112" s="12" t="n">
-        <v>45923</v>
+        <v>46118</v>
       </c>
       <c r="L112" s="13" t="n">
         <f aca="false">IF(K112="","",K112-Resumo!$B$3)</f>
-        <v>-395</v>
+        <v>-200</v>
       </c>
       <c r="M112" s="10" t="s">
         <v>267</v>
@@ -7765,7 +7786,7 @@
         <v>112</v>
       </c>
       <c r="B113" s="11" t="s">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="C113" s="10" t="s">
         <v>263</v>
@@ -7780,26 +7801,24 @@
         <v>266</v>
       </c>
       <c r="G113" s="12" t="n">
-        <v>46043</v>
+        <v>46238</v>
       </c>
       <c r="H113" s="10" t="s">
         <v>14</v>
       </c>
       <c r="I113" s="10" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J113" s="10" t="s">
-        <v>56</v>
-      </c>
-      <c r="K113" s="12" t="n">
-        <v>46113</v>
-      </c>
-      <c r="L113" s="13" t="n">
+        <v>6</v>
+      </c>
+      <c r="K113" s="12"/>
+      <c r="L113" s="13" t="str">
         <f aca="false">IF(K113="","",K113-Resumo!$B$3)</f>
-        <v>-205</v>
+        <v/>
       </c>
       <c r="M113" s="10" t="s">
-        <v>268</v>
+        <v>79</v>
       </c>
       <c r="N113" s="10" t="s">
         <v>54</v>
@@ -7811,7 +7830,7 @@
       <c r="Q113" s="15"/>
       <c r="R113" s="14"/>
     </row>
-    <row r="114" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="114" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A114" s="10" t="n">
         <v>113</v>
       </c>
@@ -7831,26 +7850,26 @@
         <v>266</v>
       </c>
       <c r="G114" s="12" t="n">
-        <v>46043</v>
+        <v>46238</v>
       </c>
       <c r="H114" s="10" t="s">
         <v>15</v>
       </c>
       <c r="I114" s="10" t="n">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="J114" s="10" t="s">
         <v>56</v>
       </c>
       <c r="K114" s="12" t="n">
-        <v>45351</v>
+        <v>46280</v>
       </c>
       <c r="L114" s="13" t="n">
         <f aca="false">IF(K114="","",K114-Resumo!$B$3)</f>
-        <v>-967</v>
+        <v>-38</v>
       </c>
       <c r="M114" s="10" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="N114" s="10" t="s">
         <v>58</v>
@@ -7867,44 +7886,44 @@
         <v>114</v>
       </c>
       <c r="B115" s="11" t="s">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="C115" s="10" t="s">
-        <v>270</v>
+        <v>263</v>
       </c>
       <c r="D115" s="10" t="s">
-        <v>207</v>
+        <v>264</v>
       </c>
       <c r="E115" s="10" t="s">
-        <v>271</v>
+        <v>265</v>
       </c>
       <c r="F115" s="10" t="s">
-        <v>272</v>
+        <v>266</v>
       </c>
       <c r="G115" s="12" t="n">
-        <v>46408</v>
+        <v>46238</v>
       </c>
       <c r="H115" s="10" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="I115" s="10" t="n">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="J115" s="10" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="K115" s="12" t="n">
-        <v>46288</v>
+        <v>46340</v>
       </c>
       <c r="L115" s="13" t="n">
         <f aca="false">IF(K115="","",K115-Resumo!$B$3)</f>
-        <v>-30</v>
+        <v>22</v>
       </c>
       <c r="M115" s="10" t="s">
-        <v>273</v>
+        <v>269</v>
       </c>
       <c r="N115" s="10" t="s">
-        <v>99</v>
+        <v>90</v>
       </c>
       <c r="O115" s="14"/>
       <c r="P115" s="14" t="s">
@@ -7913,7 +7932,7 @@
       <c r="Q115" s="15"/>
       <c r="R115" s="14"/>
     </row>
-    <row r="116" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="116" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A116" s="10" t="n">
         <v>115</v>
       </c>
@@ -7924,38 +7943,38 @@
         <v>270</v>
       </c>
       <c r="D116" s="10" t="s">
-        <v>207</v>
+        <v>271</v>
       </c>
       <c r="E116" s="10" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="F116" s="10" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="G116" s="12" t="n">
-        <v>46408</v>
+        <v>46043</v>
       </c>
       <c r="H116" s="10" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="I116" s="10" t="n">
-        <v>5</v>
+        <v>21</v>
       </c>
       <c r="J116" s="10" t="s">
         <v>56</v>
       </c>
       <c r="K116" s="12" t="n">
-        <v>46113</v>
+        <v>45923</v>
       </c>
       <c r="L116" s="13" t="n">
         <f aca="false">IF(K116="","",K116-Resumo!$B$3)</f>
-        <v>-205</v>
+        <v>-395</v>
       </c>
       <c r="M116" s="10" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
       <c r="N116" s="10" t="s">
-        <v>54</v>
+        <v>99</v>
       </c>
       <c r="O116" s="14"/>
       <c r="P116" s="14" t="s">
@@ -7964,7 +7983,7 @@
       <c r="Q116" s="15"/>
       <c r="R116" s="14"/>
     </row>
-    <row r="117" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="117" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A117" s="10" t="n">
         <v>116</v>
       </c>
@@ -7975,38 +7994,38 @@
         <v>270</v>
       </c>
       <c r="D117" s="10" t="s">
-        <v>207</v>
+        <v>271</v>
       </c>
       <c r="E117" s="10" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="F117" s="10" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="G117" s="12" t="n">
-        <v>46408</v>
+        <v>46043</v>
       </c>
       <c r="H117" s="10" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="I117" s="10" t="n">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="J117" s="10" t="s">
         <v>56</v>
       </c>
       <c r="K117" s="12" t="n">
-        <v>46282</v>
+        <v>46113</v>
       </c>
       <c r="L117" s="13" t="n">
         <f aca="false">IF(K117="","",K117-Resumo!$B$3)</f>
-        <v>-36</v>
+        <v>-205</v>
       </c>
       <c r="M117" s="10" t="s">
-        <v>74</v>
+        <v>275</v>
       </c>
       <c r="N117" s="10" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="O117" s="14"/>
       <c r="P117" s="14" t="s">
@@ -8020,42 +8039,44 @@
         <v>117</v>
       </c>
       <c r="B118" s="11" t="s">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="C118" s="10" t="s">
-        <v>274</v>
+        <v>270</v>
       </c>
       <c r="D118" s="10" t="s">
-        <v>95</v>
+        <v>271</v>
       </c>
       <c r="E118" s="10" t="s">
-        <v>275</v>
+        <v>272</v>
       </c>
       <c r="F118" s="10" t="s">
+        <v>273</v>
+      </c>
+      <c r="G118" s="12" t="n">
+        <v>46043</v>
+      </c>
+      <c r="H118" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="I118" s="10" t="n">
+        <v>17</v>
+      </c>
+      <c r="J118" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="K118" s="12" t="n">
+        <v>45351</v>
+      </c>
+      <c r="L118" s="13" t="n">
+        <f aca="false">IF(K118="","",K118-Resumo!$B$3)</f>
+        <v>-967</v>
+      </c>
+      <c r="M118" s="10" t="s">
         <v>276</v>
       </c>
-      <c r="G118" s="12" t="n">
-        <v>47310</v>
-      </c>
-      <c r="H118" s="10" t="s">
-        <v>13</v>
-      </c>
-      <c r="I118" s="10" t="n">
-        <v>9</v>
-      </c>
-      <c r="J118" s="10" t="s">
-        <v>6</v>
-      </c>
-      <c r="K118" s="12"/>
-      <c r="L118" s="13" t="str">
-        <f aca="false">IF(K118="","",K118-Resumo!$B$3)</f>
-        <v/>
-      </c>
-      <c r="M118" s="10" t="s">
-        <v>79</v>
-      </c>
       <c r="N118" s="10" t="s">
-        <v>162</v>
+        <v>58</v>
       </c>
       <c r="O118" s="14"/>
       <c r="P118" s="14" t="s">
@@ -8064,47 +8085,49 @@
       <c r="Q118" s="15"/>
       <c r="R118" s="14"/>
     </row>
-    <row r="119" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="119" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A119" s="10" t="n">
         <v>118</v>
       </c>
       <c r="B119" s="11" t="s">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="C119" s="10" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
       <c r="D119" s="10" t="s">
-        <v>95</v>
+        <v>207</v>
       </c>
       <c r="E119" s="10" t="s">
-        <v>275</v>
+        <v>278</v>
       </c>
       <c r="F119" s="10" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="G119" s="12" t="n">
-        <v>47310</v>
+        <v>46408</v>
       </c>
       <c r="H119" s="10" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="I119" s="10" t="n">
-        <v>5</v>
+        <v>19</v>
       </c>
       <c r="J119" s="10" t="s">
-        <v>6</v>
-      </c>
-      <c r="K119" s="12"/>
-      <c r="L119" s="13" t="str">
+        <v>56</v>
+      </c>
+      <c r="K119" s="12" t="n">
+        <v>46288</v>
+      </c>
+      <c r="L119" s="13" t="n">
         <f aca="false">IF(K119="","",K119-Resumo!$B$3)</f>
-        <v/>
+        <v>-30</v>
       </c>
       <c r="M119" s="10" t="s">
-        <v>79</v>
+        <v>280</v>
       </c>
       <c r="N119" s="10" t="s">
-        <v>54</v>
+        <v>99</v>
       </c>
       <c r="O119" s="14"/>
       <c r="P119" s="14" t="s">
@@ -8113,7 +8136,7 @@
       <c r="Q119" s="15"/>
       <c r="R119" s="14"/>
     </row>
-    <row r="120" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="120" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A120" s="10" t="n">
         <v>119</v>
       </c>
@@ -8121,41 +8144,41 @@
         <v>55</v>
       </c>
       <c r="C120" s="10" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
       <c r="D120" s="10" t="s">
-        <v>95</v>
+        <v>207</v>
       </c>
       <c r="E120" s="10" t="s">
-        <v>275</v>
+        <v>278</v>
       </c>
       <c r="F120" s="10" t="s">
-        <v>276</v>
+        <v>279</v>
       </c>
       <c r="G120" s="12" t="n">
-        <v>47310</v>
+        <v>46408</v>
       </c>
       <c r="H120" s="10" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="I120" s="10" t="n">
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="J120" s="10" t="s">
         <v>56</v>
       </c>
       <c r="K120" s="12" t="n">
-        <v>46043</v>
+        <v>46113</v>
       </c>
       <c r="L120" s="13" t="n">
         <f aca="false">IF(K120="","",K120-Resumo!$B$3)</f>
-        <v>-275</v>
+        <v>-205</v>
       </c>
       <c r="M120" s="10" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="N120" s="10" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="O120" s="14"/>
       <c r="P120" s="14" t="s">
@@ -8164,7 +8187,7 @@
       <c r="Q120" s="15"/>
       <c r="R120" s="14"/>
     </row>
-    <row r="121" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="121" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A121" s="10" t="n">
         <v>120</v>
       </c>
@@ -8172,41 +8195,41 @@
         <v>55</v>
       </c>
       <c r="C121" s="10" t="s">
+        <v>277</v>
+      </c>
+      <c r="D121" s="10" t="s">
+        <v>207</v>
+      </c>
+      <c r="E121" s="10" t="s">
         <v>278</v>
       </c>
-      <c r="D121" s="10" t="s">
-        <v>158</v>
-      </c>
-      <c r="E121" s="10" t="s">
+      <c r="F121" s="10" t="s">
         <v>279</v>
       </c>
-      <c r="F121" s="10" t="s">
-        <v>280</v>
-      </c>
       <c r="G121" s="12" t="n">
-        <v>46658</v>
+        <v>46408</v>
       </c>
       <c r="H121" s="10" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="I121" s="10" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="J121" s="10" t="s">
         <v>56</v>
       </c>
       <c r="K121" s="12" t="n">
-        <v>46107</v>
+        <v>46282</v>
       </c>
       <c r="L121" s="13" t="n">
         <f aca="false">IF(K121="","",K121-Resumo!$B$3)</f>
-        <v>-211</v>
+        <v>-36</v>
       </c>
       <c r="M121" s="10" t="s">
-        <v>281</v>
+        <v>74</v>
       </c>
       <c r="N121" s="10" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="O121" s="14"/>
       <c r="P121" s="14" t="s">
@@ -8220,44 +8243,42 @@
         <v>121</v>
       </c>
       <c r="B122" s="11" t="s">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="C122" s="10" t="s">
-        <v>278</v>
+        <v>281</v>
       </c>
       <c r="D122" s="10" t="s">
-        <v>158</v>
+        <v>95</v>
       </c>
       <c r="E122" s="10" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
       <c r="F122" s="10" t="s">
-        <v>280</v>
+        <v>283</v>
       </c>
       <c r="G122" s="12" t="n">
-        <v>46658</v>
+        <v>47310</v>
       </c>
       <c r="H122" s="10" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="I122" s="10" t="n">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="J122" s="10" t="s">
-        <v>56</v>
-      </c>
-      <c r="K122" s="12" t="n">
-        <v>46280</v>
-      </c>
-      <c r="L122" s="13" t="n">
+        <v>6</v>
+      </c>
+      <c r="K122" s="12"/>
+      <c r="L122" s="13" t="str">
         <f aca="false">IF(K122="","",K122-Resumo!$B$3)</f>
-        <v>-38</v>
+        <v/>
       </c>
       <c r="M122" s="10" t="s">
-        <v>231</v>
+        <v>79</v>
       </c>
       <c r="N122" s="10" t="s">
-        <v>58</v>
+        <v>162</v>
       </c>
       <c r="O122" s="14"/>
       <c r="P122" s="14" t="s">
@@ -8266,7 +8287,7 @@
       <c r="Q122" s="15"/>
       <c r="R122" s="14"/>
     </row>
-    <row r="123" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="123" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A123" s="10" t="n">
         <v>122</v>
       </c>
@@ -8274,25 +8295,25 @@
         <v>45</v>
       </c>
       <c r="C123" s="10" t="s">
-        <v>278</v>
+        <v>281</v>
       </c>
       <c r="D123" s="10" t="s">
-        <v>158</v>
+        <v>95</v>
       </c>
       <c r="E123" s="10" t="s">
-        <v>279</v>
+        <v>282</v>
       </c>
       <c r="F123" s="10" t="s">
-        <v>280</v>
+        <v>283</v>
       </c>
       <c r="G123" s="12" t="n">
-        <v>46658</v>
+        <v>47310</v>
       </c>
       <c r="H123" s="10" t="s">
-        <v>19</v>
+        <v>14</v>
       </c>
       <c r="I123" s="10" t="n">
-        <v>17</v>
+        <v>5</v>
       </c>
       <c r="J123" s="10" t="s">
         <v>6</v>
@@ -8306,7 +8327,7 @@
         <v>79</v>
       </c>
       <c r="N123" s="10" t="s">
-        <v>138</v>
+        <v>54</v>
       </c>
       <c r="O123" s="14"/>
       <c r="P123" s="14" t="s">
@@ -8315,7 +8336,7 @@
       <c r="Q123" s="15"/>
       <c r="R123" s="14"/>
     </row>
-    <row r="124" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="124" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A124" s="10" t="n">
         <v>123</v>
       </c>
@@ -8323,41 +8344,41 @@
         <v>55</v>
       </c>
       <c r="C124" s="10" t="s">
+        <v>281</v>
+      </c>
+      <c r="D124" s="10" t="s">
+        <v>95</v>
+      </c>
+      <c r="E124" s="10" t="s">
         <v>282</v>
       </c>
-      <c r="D124" s="10" t="s">
+      <c r="F124" s="10" t="s">
         <v>283</v>
       </c>
-      <c r="E124" s="10" t="s">
-        <v>284</v>
-      </c>
-      <c r="F124" s="10" t="s">
-        <v>285</v>
-      </c>
       <c r="G124" s="12" t="n">
-        <v>47016</v>
+        <v>47310</v>
       </c>
       <c r="H124" s="10" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="I124" s="10" t="n">
-        <v>5</v>
+        <v>16</v>
       </c>
       <c r="J124" s="10" t="s">
         <v>56</v>
       </c>
       <c r="K124" s="12" t="n">
-        <v>46113</v>
+        <v>46043</v>
       </c>
       <c r="L124" s="13" t="n">
         <f aca="false">IF(K124="","",K124-Resumo!$B$3)</f>
-        <v>-205</v>
+        <v>-275</v>
       </c>
       <c r="M124" s="10" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="N124" s="10" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="O124" s="14"/>
       <c r="P124" s="14" t="s">
@@ -8366,7 +8387,7 @@
       <c r="Q124" s="15"/>
       <c r="R124" s="14"/>
     </row>
-    <row r="125" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="125" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A125" s="10" t="n">
         <v>124</v>
       </c>
@@ -8374,41 +8395,41 @@
         <v>55</v>
       </c>
       <c r="C125" s="10" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
       <c r="D125" s="10" t="s">
-        <v>283</v>
+        <v>158</v>
       </c>
       <c r="E125" s="10" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="F125" s="10" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="G125" s="12" t="n">
-        <v>47016</v>
+        <v>46658</v>
       </c>
       <c r="H125" s="10" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="I125" s="10" t="n">
-        <v>16</v>
+        <v>5</v>
       </c>
       <c r="J125" s="10" t="s">
         <v>56</v>
       </c>
       <c r="K125" s="12" t="n">
-        <v>45519</v>
+        <v>46107</v>
       </c>
       <c r="L125" s="13" t="n">
         <f aca="false">IF(K125="","",K125-Resumo!$B$3)</f>
-        <v>-799</v>
+        <v>-211</v>
       </c>
       <c r="M125" s="10" t="s">
-        <v>287</v>
+        <v>288</v>
       </c>
       <c r="N125" s="10" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="O125" s="14"/>
       <c r="P125" s="14" t="s">
@@ -8422,44 +8443,44 @@
         <v>125</v>
       </c>
       <c r="B126" s="11" t="s">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="C126" s="10" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
       <c r="D126" s="10" t="s">
-        <v>283</v>
+        <v>158</v>
       </c>
       <c r="E126" s="10" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="F126" s="10" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
       <c r="G126" s="12" t="n">
-        <v>47016</v>
+        <v>46658</v>
       </c>
       <c r="H126" s="10" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="I126" s="10" t="n">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="J126" s="10" t="s">
-        <v>50</v>
+        <v>56</v>
       </c>
       <c r="K126" s="12" t="n">
-        <v>46339</v>
+        <v>46280</v>
       </c>
       <c r="L126" s="13" t="n">
         <f aca="false">IF(K126="","",K126-Resumo!$B$3)</f>
-        <v>21</v>
+        <v>-38</v>
       </c>
       <c r="M126" s="10" t="s">
-        <v>288</v>
+        <v>231</v>
       </c>
       <c r="N126" s="10" t="s">
-        <v>90</v>
+        <v>58</v>
       </c>
       <c r="O126" s="14"/>
       <c r="P126" s="14" t="s">
@@ -8473,44 +8494,42 @@
         <v>126</v>
       </c>
       <c r="B127" s="11" t="s">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="C127" s="10" t="s">
-        <v>289</v>
+        <v>285</v>
       </c>
       <c r="D127" s="10" t="s">
-        <v>290</v>
+        <v>158</v>
       </c>
       <c r="E127" s="10" t="s">
-        <v>291</v>
+        <v>286</v>
       </c>
       <c r="F127" s="10" t="s">
-        <v>292</v>
+        <v>287</v>
       </c>
       <c r="G127" s="12" t="n">
-        <v>46332</v>
+        <v>46658</v>
       </c>
       <c r="H127" s="10" t="s">
-        <v>9</v>
+        <v>19</v>
       </c>
       <c r="I127" s="10" t="n">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="J127" s="10" t="s">
-        <v>56</v>
-      </c>
-      <c r="K127" s="12" t="n">
-        <v>46212</v>
-      </c>
-      <c r="L127" s="13" t="n">
+        <v>6</v>
+      </c>
+      <c r="K127" s="12"/>
+      <c r="L127" s="13" t="str">
         <f aca="false">IF(K127="","",K127-Resumo!$B$3)</f>
-        <v>-106</v>
+        <v/>
       </c>
       <c r="M127" s="10" t="s">
-        <v>293</v>
+        <v>79</v>
       </c>
       <c r="N127" s="10" t="s">
-        <v>99</v>
+        <v>138</v>
       </c>
       <c r="O127" s="14"/>
       <c r="P127" s="14" t="s">
@@ -8519,12 +8538,12 @@
       <c r="Q127" s="15"/>
       <c r="R127" s="14"/>
     </row>
-    <row r="128" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="128" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A128" s="10" t="n">
         <v>127</v>
       </c>
       <c r="B128" s="11" t="s">
-        <v>80</v>
+        <v>55</v>
       </c>
       <c r="C128" s="10" t="s">
         <v>289</v>
@@ -8539,29 +8558,29 @@
         <v>292</v>
       </c>
       <c r="G128" s="12" t="n">
-        <v>46332</v>
+        <v>47016</v>
       </c>
       <c r="H128" s="10" t="s">
-        <v>11</v>
+        <v>14</v>
       </c>
       <c r="I128" s="10" t="n">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="J128" s="10" t="s">
         <v>56</v>
       </c>
       <c r="K128" s="12" t="n">
-        <v>46248</v>
+        <v>46113</v>
       </c>
       <c r="L128" s="13" t="n">
         <f aca="false">IF(K128="","",K128-Resumo!$B$3)</f>
-        <v>-70</v>
+        <v>-205</v>
       </c>
       <c r="M128" s="10" t="s">
-        <v>85</v>
+        <v>293</v>
       </c>
       <c r="N128" s="10" t="s">
-        <v>86</v>
+        <v>54</v>
       </c>
       <c r="O128" s="14"/>
       <c r="P128" s="14" t="s">
@@ -8570,7 +8589,7 @@
       <c r="Q128" s="15"/>
       <c r="R128" s="14"/>
     </row>
-    <row r="129" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="129" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A129" s="10" t="n">
         <v>128</v>
       </c>
@@ -8590,29 +8609,29 @@
         <v>292</v>
       </c>
       <c r="G129" s="12" t="n">
-        <v>46332</v>
+        <v>47016</v>
       </c>
       <c r="H129" s="10" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="I129" s="10" t="n">
         <v>16</v>
       </c>
       <c r="J129" s="10" t="s">
-        <v>50</v>
+        <v>56</v>
       </c>
       <c r="K129" s="12" t="n">
-        <v>46328</v>
+        <v>45519</v>
       </c>
       <c r="L129" s="13" t="n">
         <f aca="false">IF(K129="","",K129-Resumo!$B$3)</f>
-        <v>10</v>
+        <v>-799</v>
       </c>
       <c r="M129" s="10" t="s">
-        <v>87</v>
+        <v>294</v>
       </c>
       <c r="N129" s="10" t="s">
-        <v>88</v>
+        <v>58</v>
       </c>
       <c r="O129" s="14"/>
       <c r="P129" s="14" t="s">
@@ -8621,12 +8640,12 @@
       <c r="Q129" s="15"/>
       <c r="R129" s="14"/>
     </row>
-    <row r="130" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="130" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A130" s="10" t="n">
         <v>129</v>
       </c>
       <c r="B130" s="11" t="s">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="C130" s="10" t="s">
         <v>289</v>
@@ -8641,29 +8660,29 @@
         <v>292</v>
       </c>
       <c r="G130" s="12" t="n">
-        <v>46332</v>
+        <v>47016</v>
       </c>
       <c r="H130" s="10" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="I130" s="10" t="n">
-        <v>5</v>
+        <v>15</v>
       </c>
       <c r="J130" s="10" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="K130" s="12" t="n">
-        <v>46259</v>
+        <v>46339</v>
       </c>
       <c r="L130" s="13" t="n">
         <f aca="false">IF(K130="","",K130-Resumo!$B$3)</f>
-        <v>-59</v>
+        <v>21</v>
       </c>
       <c r="M130" s="10" t="s">
-        <v>294</v>
+        <v>295</v>
       </c>
       <c r="N130" s="10" t="s">
-        <v>54</v>
+        <v>90</v>
       </c>
       <c r="O130" s="14"/>
       <c r="P130" s="14" t="s">
@@ -8680,41 +8699,41 @@
         <v>55</v>
       </c>
       <c r="C131" s="10" t="s">
-        <v>289</v>
+        <v>296</v>
       </c>
       <c r="D131" s="10" t="s">
-        <v>290</v>
+        <v>297</v>
       </c>
       <c r="E131" s="10" t="s">
-        <v>291</v>
+        <v>298</v>
       </c>
       <c r="F131" s="10" t="s">
-        <v>292</v>
+        <v>299</v>
       </c>
       <c r="G131" s="12" t="n">
         <v>46332</v>
       </c>
       <c r="H131" s="10" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
       <c r="I131" s="10" t="n">
-        <v>14</v>
+        <v>19</v>
       </c>
       <c r="J131" s="10" t="s">
         <v>56</v>
       </c>
       <c r="K131" s="12" t="n">
-        <v>46280</v>
+        <v>46212</v>
       </c>
       <c r="L131" s="13" t="n">
         <f aca="false">IF(K131="","",K131-Resumo!$B$3)</f>
-        <v>-38</v>
+        <v>-106</v>
       </c>
       <c r="M131" s="10" t="s">
-        <v>231</v>
+        <v>300</v>
       </c>
       <c r="N131" s="10" t="s">
-        <v>58</v>
+        <v>99</v>
       </c>
       <c r="O131" s="14"/>
       <c r="P131" s="14" t="s">
@@ -8728,42 +8747,44 @@
         <v>131</v>
       </c>
       <c r="B132" s="11" t="s">
-        <v>45</v>
+        <v>80</v>
       </c>
       <c r="C132" s="10" t="s">
-        <v>289</v>
+        <v>296</v>
       </c>
       <c r="D132" s="10" t="s">
-        <v>290</v>
+        <v>297</v>
       </c>
       <c r="E132" s="10" t="s">
-        <v>291</v>
+        <v>298</v>
       </c>
       <c r="F132" s="10" t="s">
-        <v>292</v>
+        <v>299</v>
       </c>
       <c r="G132" s="12" t="n">
         <v>46332</v>
       </c>
       <c r="H132" s="10" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="I132" s="10" t="n">
-        <v>13</v>
+        <v>18</v>
       </c>
       <c r="J132" s="10" t="s">
-        <v>6</v>
-      </c>
-      <c r="K132" s="12"/>
-      <c r="L132" s="13" t="str">
+        <v>56</v>
+      </c>
+      <c r="K132" s="12" t="n">
+        <v>46248</v>
+      </c>
+      <c r="L132" s="13" t="n">
         <f aca="false">IF(K132="","",K132-Resumo!$B$3)</f>
-        <v/>
+        <v>-70</v>
       </c>
       <c r="M132" s="10" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="N132" s="10" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="O132" s="14"/>
       <c r="P132" s="14" t="s">
@@ -8772,49 +8793,49 @@
       <c r="Q132" s="15"/>
       <c r="R132" s="14"/>
     </row>
-    <row r="133" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="133" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A133" s="10" t="n">
         <v>132</v>
       </c>
       <c r="B133" s="11" t="s">
-        <v>80</v>
+        <v>55</v>
       </c>
       <c r="C133" s="10" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="D133" s="10" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="E133" s="10" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="F133" s="10" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="G133" s="12" t="n">
-        <v>48215</v>
+        <v>46332</v>
       </c>
       <c r="H133" s="10" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="I133" s="10" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="J133" s="10" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="K133" s="12" t="n">
-        <v>46034</v>
+        <v>46328</v>
       </c>
       <c r="L133" s="13" t="n">
         <f aca="false">IF(K133="","",K133-Resumo!$B$3)</f>
-        <v>-284</v>
+        <v>10</v>
       </c>
       <c r="M133" s="10" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="N133" s="10" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="O133" s="14"/>
       <c r="P133" s="14" t="s">
@@ -8823,49 +8844,49 @@
       <c r="Q133" s="15"/>
       <c r="R133" s="14"/>
     </row>
-    <row r="134" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="134" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A134" s="10" t="n">
         <v>133</v>
       </c>
       <c r="B134" s="11" t="s">
-        <v>80</v>
+        <v>55</v>
       </c>
       <c r="C134" s="10" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="D134" s="10" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="E134" s="10" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="F134" s="10" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="G134" s="12" t="n">
-        <v>48215</v>
+        <v>46332</v>
       </c>
       <c r="H134" s="10" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="I134" s="10" t="n">
-        <v>18</v>
+        <v>5</v>
       </c>
       <c r="J134" s="10" t="s">
         <v>56</v>
       </c>
       <c r="K134" s="12" t="n">
-        <v>46114</v>
+        <v>46259</v>
       </c>
       <c r="L134" s="13" t="n">
         <f aca="false">IF(K134="","",K134-Resumo!$B$3)</f>
-        <v>-204</v>
+        <v>-59</v>
       </c>
       <c r="M134" s="10" t="s">
-        <v>87</v>
+        <v>301</v>
       </c>
       <c r="N134" s="10" t="s">
-        <v>88</v>
+        <v>54</v>
       </c>
       <c r="O134" s="14"/>
       <c r="P134" s="14" t="s">
@@ -8874,7 +8895,7 @@
       <c r="Q134" s="15"/>
       <c r="R134" s="14"/>
     </row>
-    <row r="135" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="135" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A135" s="10" t="n">
         <v>134</v>
       </c>
@@ -8882,41 +8903,41 @@
         <v>55</v>
       </c>
       <c r="C135" s="10" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="D135" s="10" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="E135" s="10" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="F135" s="10" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="G135" s="12" t="n">
-        <v>48215</v>
+        <v>46332</v>
       </c>
       <c r="H135" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="I135" s="10" t="n">
         <v>14</v>
-      </c>
-      <c r="I135" s="10" t="n">
-        <v>5</v>
       </c>
       <c r="J135" s="10" t="s">
         <v>56</v>
       </c>
       <c r="K135" s="12" t="n">
-        <v>46276</v>
+        <v>46280</v>
       </c>
       <c r="L135" s="13" t="n">
         <f aca="false">IF(K135="","",K135-Resumo!$B$3)</f>
-        <v>-42</v>
+        <v>-38</v>
       </c>
       <c r="M135" s="10" t="s">
-        <v>299</v>
+        <v>231</v>
       </c>
       <c r="N135" s="10" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="O135" s="14"/>
       <c r="P135" s="14" t="s">
@@ -8933,25 +8954,25 @@
         <v>45</v>
       </c>
       <c r="C136" s="10" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="D136" s="10" t="s">
-        <v>296</v>
+        <v>297</v>
       </c>
       <c r="E136" s="10" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="F136" s="10" t="s">
-        <v>298</v>
+        <v>299</v>
       </c>
       <c r="G136" s="12" t="n">
-        <v>48215</v>
+        <v>46332</v>
       </c>
       <c r="H136" s="10" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="I136" s="10" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="J136" s="10" t="s">
         <v>6</v>
@@ -8965,7 +8986,7 @@
         <v>79</v>
       </c>
       <c r="N136" s="10" t="s">
-        <v>58</v>
+        <v>90</v>
       </c>
       <c r="O136" s="14"/>
       <c r="P136" s="14" t="s">
@@ -8979,42 +9000,44 @@
         <v>136</v>
       </c>
       <c r="B137" s="11" t="s">
-        <v>45</v>
+        <v>80</v>
       </c>
       <c r="C137" s="10" t="s">
-        <v>295</v>
+        <v>302</v>
       </c>
       <c r="D137" s="10" t="s">
-        <v>296</v>
+        <v>303</v>
       </c>
       <c r="E137" s="10" t="s">
-        <v>297</v>
+        <v>304</v>
       </c>
       <c r="F137" s="10" t="s">
-        <v>298</v>
+        <v>305</v>
       </c>
       <c r="G137" s="12" t="n">
         <v>48215</v>
       </c>
       <c r="H137" s="10" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="I137" s="10" t="n">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="J137" s="10" t="s">
-        <v>6</v>
-      </c>
-      <c r="K137" s="12"/>
-      <c r="L137" s="13" t="str">
+        <v>56</v>
+      </c>
+      <c r="K137" s="12" t="n">
+        <v>46034</v>
+      </c>
+      <c r="L137" s="13" t="n">
         <f aca="false">IF(K137="","",K137-Resumo!$B$3)</f>
-        <v/>
+        <v>-284</v>
       </c>
       <c r="M137" s="10" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="N137" s="10" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="O137" s="14"/>
       <c r="P137" s="14" t="s">
@@ -9023,47 +9046,49 @@
       <c r="Q137" s="15"/>
       <c r="R137" s="14"/>
     </row>
-    <row r="138" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="138" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A138" s="10" t="n">
         <v>137</v>
       </c>
       <c r="B138" s="11" t="s">
-        <v>45</v>
+        <v>80</v>
       </c>
       <c r="C138" s="10" t="s">
-        <v>295</v>
+        <v>302</v>
       </c>
       <c r="D138" s="10" t="s">
-        <v>296</v>
+        <v>303</v>
       </c>
       <c r="E138" s="10" t="s">
-        <v>297</v>
+        <v>304</v>
       </c>
       <c r="F138" s="10" t="s">
-        <v>298</v>
+        <v>305</v>
       </c>
       <c r="G138" s="12" t="n">
         <v>48215</v>
       </c>
       <c r="H138" s="10" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="I138" s="10" t="n">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="J138" s="10" t="s">
-        <v>6</v>
-      </c>
-      <c r="K138" s="12"/>
-      <c r="L138" s="13" t="str">
+        <v>56</v>
+      </c>
+      <c r="K138" s="12" t="n">
+        <v>46114</v>
+      </c>
+      <c r="L138" s="13" t="n">
         <f aca="false">IF(K138="","",K138-Resumo!$B$3)</f>
-        <v/>
+        <v>-204</v>
       </c>
       <c r="M138" s="10" t="s">
-        <v>79</v>
+        <v>87</v>
       </c>
       <c r="N138" s="10" t="s">
-        <v>92</v>
+        <v>88</v>
       </c>
       <c r="O138" s="14"/>
       <c r="P138" s="14" t="s">
@@ -9072,47 +9097,49 @@
       <c r="Q138" s="15"/>
       <c r="R138" s="14"/>
     </row>
-    <row r="139" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="139" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A139" s="10" t="n">
         <v>138</v>
       </c>
       <c r="B139" s="11" t="s">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="C139" s="10" t="s">
-        <v>295</v>
+        <v>302</v>
       </c>
       <c r="D139" s="10" t="s">
-        <v>296</v>
+        <v>303</v>
       </c>
       <c r="E139" s="10" t="s">
-        <v>297</v>
+        <v>304</v>
       </c>
       <c r="F139" s="10" t="s">
-        <v>298</v>
+        <v>305</v>
       </c>
       <c r="G139" s="12" t="n">
         <v>48215</v>
       </c>
       <c r="H139" s="10" t="s">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="I139" s="10" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="J139" s="10" t="s">
-        <v>6</v>
-      </c>
-      <c r="K139" s="12"/>
-      <c r="L139" s="13" t="str">
+        <v>56</v>
+      </c>
+      <c r="K139" s="12" t="n">
+        <v>46276</v>
+      </c>
+      <c r="L139" s="13" t="n">
         <f aca="false">IF(K139="","",K139-Resumo!$B$3)</f>
-        <v/>
+        <v>-42</v>
       </c>
       <c r="M139" s="10" t="s">
-        <v>79</v>
+        <v>306</v>
       </c>
       <c r="N139" s="10" t="s">
-        <v>93</v>
+        <v>54</v>
       </c>
       <c r="O139" s="14"/>
       <c r="P139" s="14" t="s">
@@ -9129,39 +9156,39 @@
         <v>45</v>
       </c>
       <c r="C140" s="10" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="D140" s="10" t="s">
-        <v>198</v>
+        <v>303</v>
       </c>
       <c r="E140" s="10" t="s">
-        <v>301</v>
+        <v>304</v>
       </c>
       <c r="F140" s="10" t="s">
-        <v>302</v>
+        <v>305</v>
       </c>
       <c r="G140" s="12" t="n">
-        <v>47697</v>
+        <v>48215</v>
       </c>
       <c r="H140" s="10" t="s">
-        <v>10</v>
-      </c>
-      <c r="I140" s="10"/>
+        <v>15</v>
+      </c>
+      <c r="I140" s="10" t="n">
+        <v>15</v>
+      </c>
       <c r="J140" s="10" t="s">
-        <v>50</v>
-      </c>
-      <c r="K140" s="12" t="n">
-        <v>46344</v>
-      </c>
-      <c r="L140" s="13" t="n">
+        <v>6</v>
+      </c>
+      <c r="K140" s="12"/>
+      <c r="L140" s="13" t="str">
         <f aca="false">IF(K140="","",K140-Resumo!$B$3)</f>
-        <v>26</v>
+        <v/>
       </c>
       <c r="M140" s="10" t="s">
-        <v>51</v>
+        <v>79</v>
       </c>
       <c r="N140" s="10" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="O140" s="14"/>
       <c r="P140" s="14" t="s">
@@ -9170,49 +9197,47 @@
       <c r="Q140" s="15"/>
       <c r="R140" s="14"/>
     </row>
-    <row r="141" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="141" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A141" s="10" t="n">
         <v>140</v>
       </c>
       <c r="B141" s="11" t="s">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="C141" s="10" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="D141" s="10" t="s">
-        <v>198</v>
+        <v>303</v>
       </c>
       <c r="E141" s="10" t="s">
-        <v>301</v>
+        <v>304</v>
       </c>
       <c r="F141" s="10" t="s">
-        <v>302</v>
+        <v>305</v>
       </c>
       <c r="G141" s="12" t="n">
-        <v>47697</v>
+        <v>48215</v>
       </c>
       <c r="H141" s="10" t="s">
+        <v>16</v>
+      </c>
+      <c r="I141" s="10" t="n">
         <v>14</v>
       </c>
-      <c r="I141" s="10" t="n">
-        <v>5</v>
-      </c>
       <c r="J141" s="10" t="s">
-        <v>56</v>
-      </c>
-      <c r="K141" s="12" t="n">
-        <v>46127</v>
-      </c>
-      <c r="L141" s="13" t="n">
+        <v>6</v>
+      </c>
+      <c r="K141" s="12"/>
+      <c r="L141" s="13" t="str">
         <f aca="false">IF(K141="","",K141-Resumo!$B$3)</f>
-        <v>-191</v>
+        <v/>
       </c>
       <c r="M141" s="10" t="s">
-        <v>262</v>
+        <v>79</v>
       </c>
       <c r="N141" s="10" t="s">
-        <v>54</v>
+        <v>90</v>
       </c>
       <c r="O141" s="14"/>
       <c r="P141" s="14" t="s">
@@ -9226,44 +9251,42 @@
         <v>141</v>
       </c>
       <c r="B142" s="11" t="s">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="C142" s="10" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="D142" s="10" t="s">
-        <v>198</v>
+        <v>303</v>
       </c>
       <c r="E142" s="10" t="s">
-        <v>301</v>
+        <v>304</v>
       </c>
       <c r="F142" s="10" t="s">
-        <v>302</v>
+        <v>305</v>
       </c>
       <c r="G142" s="12" t="n">
-        <v>47697</v>
+        <v>48215</v>
       </c>
       <c r="H142" s="10" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="I142" s="10" t="n">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="J142" s="10" t="s">
-        <v>56</v>
-      </c>
-      <c r="K142" s="12" t="n">
-        <v>46282</v>
-      </c>
-      <c r="L142" s="13" t="n">
+        <v>6</v>
+      </c>
+      <c r="K142" s="12"/>
+      <c r="L142" s="13" t="str">
         <f aca="false">IF(K142="","",K142-Resumo!$B$3)</f>
-        <v>-36</v>
+        <v/>
       </c>
       <c r="M142" s="10" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="N142" s="10" t="s">
-        <v>58</v>
+        <v>92</v>
       </c>
       <c r="O142" s="14"/>
       <c r="P142" s="14" t="s">
@@ -9277,44 +9300,42 @@
         <v>142</v>
       </c>
       <c r="B143" s="11" t="s">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="C143" s="10" t="s">
+        <v>302</v>
+      </c>
+      <c r="D143" s="10" t="s">
         <v>303</v>
       </c>
-      <c r="D143" s="10" t="s">
+      <c r="E143" s="10" t="s">
         <v>304</v>
       </c>
-      <c r="E143" s="10" t="s">
+      <c r="F143" s="10" t="s">
         <v>305</v>
       </c>
-      <c r="F143" s="10" t="s">
-        <v>306</v>
-      </c>
       <c r="G143" s="12" t="n">
-        <v>46244</v>
+        <v>48215</v>
       </c>
       <c r="H143" s="10" t="s">
-        <v>9</v>
+        <v>18</v>
       </c>
       <c r="I143" s="10" t="n">
-        <v>21</v>
+        <v>8</v>
       </c>
       <c r="J143" s="10" t="s">
-        <v>56</v>
-      </c>
-      <c r="K143" s="12" t="n">
-        <v>46124</v>
-      </c>
-      <c r="L143" s="13" t="n">
+        <v>6</v>
+      </c>
+      <c r="K143" s="12"/>
+      <c r="L143" s="13" t="str">
         <f aca="false">IF(K143="","",K143-Resumo!$B$3)</f>
-        <v>-194</v>
+        <v/>
       </c>
       <c r="M143" s="10" t="s">
-        <v>307</v>
+        <v>79</v>
       </c>
       <c r="N143" s="10" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="O143" s="14"/>
       <c r="P143" s="14" t="s">
@@ -9323,49 +9344,47 @@
       <c r="Q143" s="15"/>
       <c r="R143" s="14"/>
     </row>
-    <row r="144" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="144" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A144" s="10" t="n">
         <v>143</v>
       </c>
       <c r="B144" s="11" t="s">
-        <v>55</v>
+        <v>45</v>
       </c>
       <c r="C144" s="10" t="s">
-        <v>303</v>
+        <v>307</v>
       </c>
       <c r="D144" s="10" t="s">
-        <v>304</v>
+        <v>198</v>
       </c>
       <c r="E144" s="10" t="s">
-        <v>305</v>
+        <v>308</v>
       </c>
       <c r="F144" s="10" t="s">
-        <v>306</v>
+        <v>309</v>
       </c>
       <c r="G144" s="12" t="n">
-        <v>46244</v>
+        <v>47697</v>
       </c>
       <c r="H144" s="10" t="s">
-        <v>14</v>
-      </c>
-      <c r="I144" s="10" t="n">
-        <v>5</v>
-      </c>
+        <v>10</v>
+      </c>
+      <c r="I144" s="10"/>
       <c r="J144" s="10" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="K144" s="12" t="n">
-        <v>46276</v>
+        <v>46344</v>
       </c>
       <c r="L144" s="13" t="n">
         <f aca="false">IF(K144="","",K144-Resumo!$B$3)</f>
-        <v>-42</v>
+        <v>26</v>
       </c>
       <c r="M144" s="10" t="s">
-        <v>299</v>
+        <v>51</v>
       </c>
       <c r="N144" s="10" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="O144" s="14"/>
       <c r="P144" s="14" t="s">
@@ -9374,47 +9393,49 @@
       <c r="Q144" s="15"/>
       <c r="R144" s="14"/>
     </row>
-    <row r="145" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="145" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A145" s="10" t="n">
         <v>144</v>
       </c>
       <c r="B145" s="11" t="s">
-        <v>45</v>
+        <v>55</v>
       </c>
       <c r="C145" s="10" t="s">
-        <v>303</v>
+        <v>307</v>
       </c>
       <c r="D145" s="10" t="s">
-        <v>304</v>
+        <v>198</v>
       </c>
       <c r="E145" s="10" t="s">
-        <v>305</v>
+        <v>308</v>
       </c>
       <c r="F145" s="10" t="s">
-        <v>306</v>
+        <v>309</v>
       </c>
       <c r="G145" s="12" t="n">
-        <v>46244</v>
+        <v>47697</v>
       </c>
       <c r="H145" s="10" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="I145" s="10" t="n">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="J145" s="10" t="s">
-        <v>6</v>
-      </c>
-      <c r="K145" s="12"/>
-      <c r="L145" s="13" t="str">
+        <v>56</v>
+      </c>
+      <c r="K145" s="12" t="n">
+        <v>46127</v>
+      </c>
+      <c r="L145" s="13" t="n">
         <f aca="false">IF(K145="","",K145-Resumo!$B$3)</f>
-        <v/>
+        <v>-191</v>
       </c>
       <c r="M145" s="10" t="s">
-        <v>79</v>
+        <v>262</v>
       </c>
       <c r="N145" s="10" t="s">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="O145" s="14"/>
       <c r="P145" s="14" t="s">
@@ -9423,9 +9444,211 @@
       <c r="Q145" s="15"/>
       <c r="R145" s="14"/>
     </row>
+    <row r="146" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A146" s="10" t="n">
+        <v>145</v>
+      </c>
+      <c r="B146" s="11" t="s">
+        <v>55</v>
+      </c>
+      <c r="C146" s="10" t="s">
+        <v>307</v>
+      </c>
+      <c r="D146" s="10" t="s">
+        <v>198</v>
+      </c>
+      <c r="E146" s="10" t="s">
+        <v>308</v>
+      </c>
+      <c r="F146" s="10" t="s">
+        <v>309</v>
+      </c>
+      <c r="G146" s="12" t="n">
+        <v>47697</v>
+      </c>
+      <c r="H146" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="I146" s="10" t="n">
+        <v>17</v>
+      </c>
+      <c r="J146" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="K146" s="12" t="n">
+        <v>46282</v>
+      </c>
+      <c r="L146" s="13" t="n">
+        <f aca="false">IF(K146="","",K146-Resumo!$B$3)</f>
+        <v>-36</v>
+      </c>
+      <c r="M146" s="10" t="s">
+        <v>74</v>
+      </c>
+      <c r="N146" s="10" t="s">
+        <v>58</v>
+      </c>
+      <c r="O146" s="14"/>
+      <c r="P146" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q146" s="15"/>
+      <c r="R146" s="14"/>
+    </row>
+    <row r="147" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A147" s="10" t="n">
+        <v>146</v>
+      </c>
+      <c r="B147" s="11" t="s">
+        <v>55</v>
+      </c>
+      <c r="C147" s="10" t="s">
+        <v>310</v>
+      </c>
+      <c r="D147" s="10" t="s">
+        <v>311</v>
+      </c>
+      <c r="E147" s="10" t="s">
+        <v>312</v>
+      </c>
+      <c r="F147" s="10" t="s">
+        <v>313</v>
+      </c>
+      <c r="G147" s="12" t="n">
+        <v>46244</v>
+      </c>
+      <c r="H147" s="10" t="s">
+        <v>9</v>
+      </c>
+      <c r="I147" s="10" t="n">
+        <v>21</v>
+      </c>
+      <c r="J147" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="K147" s="12" t="n">
+        <v>46124</v>
+      </c>
+      <c r="L147" s="13" t="n">
+        <f aca="false">IF(K147="","",K147-Resumo!$B$3)</f>
+        <v>-194</v>
+      </c>
+      <c r="M147" s="10" t="s">
+        <v>314</v>
+      </c>
+      <c r="N147" s="10" t="s">
+        <v>99</v>
+      </c>
+      <c r="O147" s="14"/>
+      <c r="P147" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q147" s="15"/>
+      <c r="R147" s="14"/>
+    </row>
+    <row r="148" customFormat="false" ht="32.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A148" s="10" t="n">
+        <v>147</v>
+      </c>
+      <c r="B148" s="11" t="s">
+        <v>55</v>
+      </c>
+      <c r="C148" s="10" t="s">
+        <v>310</v>
+      </c>
+      <c r="D148" s="10" t="s">
+        <v>311</v>
+      </c>
+      <c r="E148" s="10" t="s">
+        <v>312</v>
+      </c>
+      <c r="F148" s="10" t="s">
+        <v>313</v>
+      </c>
+      <c r="G148" s="12" t="n">
+        <v>46244</v>
+      </c>
+      <c r="H148" s="10" t="s">
+        <v>14</v>
+      </c>
+      <c r="I148" s="10" t="n">
+        <v>5</v>
+      </c>
+      <c r="J148" s="10" t="s">
+        <v>56</v>
+      </c>
+      <c r="K148" s="12" t="n">
+        <v>46276</v>
+      </c>
+      <c r="L148" s="13" t="n">
+        <f aca="false">IF(K148="","",K148-Resumo!$B$3)</f>
+        <v>-42</v>
+      </c>
+      <c r="M148" s="10" t="s">
+        <v>306</v>
+      </c>
+      <c r="N148" s="10" t="s">
+        <v>54</v>
+      </c>
+      <c r="O148" s="14"/>
+      <c r="P148" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q148" s="15"/>
+      <c r="R148" s="14"/>
+    </row>
+    <row r="149" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A149" s="10" t="n">
+        <v>148</v>
+      </c>
+      <c r="B149" s="11" t="s">
+        <v>45</v>
+      </c>
+      <c r="C149" s="10" t="s">
+        <v>310</v>
+      </c>
+      <c r="D149" s="10" t="s">
+        <v>311</v>
+      </c>
+      <c r="E149" s="10" t="s">
+        <v>312</v>
+      </c>
+      <c r="F149" s="10" t="s">
+        <v>313</v>
+      </c>
+      <c r="G149" s="12" t="n">
+        <v>46244</v>
+      </c>
+      <c r="H149" s="10" t="s">
+        <v>15</v>
+      </c>
+      <c r="I149" s="10" t="n">
+        <v>15</v>
+      </c>
+      <c r="J149" s="10" t="s">
+        <v>6</v>
+      </c>
+      <c r="K149" s="12"/>
+      <c r="L149" s="13" t="str">
+        <f aca="false">IF(K149="","",K149-Resumo!$B$3)</f>
+        <v/>
+      </c>
+      <c r="M149" s="10" t="s">
+        <v>79</v>
+      </c>
+      <c r="N149" s="10" t="s">
+        <v>58</v>
+      </c>
+      <c r="O149" s="14"/>
+      <c r="P149" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="Q149" s="15"/>
+      <c r="R149" s="14"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:R145"/>
-  <conditionalFormatting sqref="J2:J145">
+  <autoFilter ref="A1:R149"/>
+  <conditionalFormatting sqref="J2:J149">
     <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="11">
       <formula>$J2="Vencida"</formula>
     </cfRule>
@@ -9436,12 +9659,12 @@
       <formula>$J2="Sem data"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="B2:B145">
+  <conditionalFormatting sqref="B2:B149">
     <cfRule type="expression" priority="5" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="14">
       <formula>$B2="Alta"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="P2:P145">
+  <conditionalFormatting sqref="P2:P149">
     <cfRule type="expression" priority="6" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="15">
       <formula>$P2="Resolvido"</formula>
     </cfRule>
@@ -9450,7 +9673,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="P2:P145" type="list">
+    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="P2:P149" type="list">
       <formula1>"A fazer,Em andamento,Aguardando cliente,Resolvido,Já estava em dia"</formula1>
       <formula2>0</formula2>
     </dataValidation>
@@ -9471,7 +9694,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F50"/>
+  <dimension ref="A1:F51"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="42"/>
@@ -9495,7 +9718,7 @@
         <v>8</v>
       </c>
       <c r="F1" s="5" t="s">
-        <v>308</v>
+        <v>315</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9503,15 +9726,15 @@
         <v>46</v>
       </c>
       <c r="B2" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A2,Pendências!$J$2:$J$145,"Vencida")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A2,Pendências!$J$2:$J$149,"Vencida")</f>
         <v>1</v>
       </c>
       <c r="C2" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A2,Pendências!$J$2:$J$145,"Sem data")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A2,Pendências!$J$2:$J$149,"Sem data")</f>
         <v>0</v>
       </c>
       <c r="D2" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A2,Pendências!$J$2:$J$145,"Vence em breve")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A2,Pendências!$J$2:$J$149,"Vence em breve")</f>
         <v>2</v>
       </c>
       <c r="E2" s="7" t="n">
@@ -9519,7 +9742,7 @@
         <v>3</v>
       </c>
       <c r="F2" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A2,Pendências!$B$2:$B$145,"Alta")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A2,Pendências!$B$2:$B$149,"Alta")</f>
         <v>1</v>
       </c>
     </row>
@@ -9528,15 +9751,15 @@
         <v>59</v>
       </c>
       <c r="B3" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A3,Pendências!$J$2:$J$145,"Vencida")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A3,Pendências!$J$2:$J$149,"Vencida")</f>
         <v>2</v>
       </c>
       <c r="C3" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A3,Pendências!$J$2:$J$145,"Sem data")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A3,Pendências!$J$2:$J$149,"Sem data")</f>
         <v>0</v>
       </c>
       <c r="D3" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A3,Pendências!$J$2:$J$145,"Vence em breve")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A3,Pendências!$J$2:$J$149,"Vence em breve")</f>
         <v>0</v>
       </c>
       <c r="E3" s="7" t="n">
@@ -9544,7 +9767,7 @@
         <v>2</v>
       </c>
       <c r="F3" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A3,Pendências!$B$2:$B$145,"Alta")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A3,Pendências!$B$2:$B$149,"Alta")</f>
         <v>2</v>
       </c>
     </row>
@@ -9553,15 +9776,15 @@
         <v>64</v>
       </c>
       <c r="B4" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A4,Pendências!$J$2:$J$145,"Vencida")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A4,Pendências!$J$2:$J$149,"Vencida")</f>
         <v>2</v>
       </c>
       <c r="C4" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A4,Pendências!$J$2:$J$145,"Sem data")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A4,Pendências!$J$2:$J$149,"Sem data")</f>
         <v>0</v>
       </c>
       <c r="D4" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A4,Pendências!$J$2:$J$145,"Vence em breve")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A4,Pendências!$J$2:$J$149,"Vence em breve")</f>
         <v>0</v>
       </c>
       <c r="E4" s="7" t="n">
@@ -9569,7 +9792,7 @@
         <v>2</v>
       </c>
       <c r="F4" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A4,Pendências!$B$2:$B$145,"Alta")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A4,Pendências!$B$2:$B$149,"Alta")</f>
         <v>2</v>
       </c>
     </row>
@@ -9578,15 +9801,15 @@
         <v>69</v>
       </c>
       <c r="B5" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A5,Pendências!$J$2:$J$145,"Vencida")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A5,Pendências!$J$2:$J$149,"Vencida")</f>
         <v>2</v>
       </c>
       <c r="C5" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A5,Pendências!$J$2:$J$145,"Sem data")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A5,Pendências!$J$2:$J$149,"Sem data")</f>
         <v>0</v>
       </c>
       <c r="D5" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A5,Pendências!$J$2:$J$145,"Vence em breve")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A5,Pendências!$J$2:$J$149,"Vence em breve")</f>
         <v>0</v>
       </c>
       <c r="E5" s="7" t="n">
@@ -9594,7 +9817,7 @@
         <v>2</v>
       </c>
       <c r="F5" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A5,Pendências!$B$2:$B$145,"Alta")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A5,Pendências!$B$2:$B$149,"Alta")</f>
         <v>2</v>
       </c>
     </row>
@@ -9603,15 +9826,15 @@
         <v>75</v>
       </c>
       <c r="B6" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A6,Pendências!$J$2:$J$145,"Vencida")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A6,Pendências!$J$2:$J$149,"Vencida")</f>
         <v>0</v>
       </c>
       <c r="C6" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A6,Pendências!$J$2:$J$145,"Sem data")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A6,Pendências!$J$2:$J$149,"Sem data")</f>
         <v>1</v>
       </c>
       <c r="D6" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A6,Pendências!$J$2:$J$145,"Vence em breve")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A6,Pendências!$J$2:$J$149,"Vence em breve")</f>
         <v>0</v>
       </c>
       <c r="E6" s="7" t="n">
@@ -9619,7 +9842,7 @@
         <v>1</v>
       </c>
       <c r="F6" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A6,Pendências!$B$2:$B$145,"Alta")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A6,Pendências!$B$2:$B$149,"Alta")</f>
         <v>0</v>
       </c>
     </row>
@@ -9628,15 +9851,15 @@
         <v>81</v>
       </c>
       <c r="B7" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A7,Pendências!$J$2:$J$145,"Vencida")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A7,Pendências!$J$2:$J$149,"Vencida")</f>
         <v>5</v>
       </c>
       <c r="C7" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A7,Pendências!$J$2:$J$145,"Sem data")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A7,Pendências!$J$2:$J$149,"Sem data")</f>
         <v>2</v>
       </c>
       <c r="D7" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A7,Pendências!$J$2:$J$145,"Vence em breve")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A7,Pendências!$J$2:$J$149,"Vence em breve")</f>
         <v>0</v>
       </c>
       <c r="E7" s="7" t="n">
@@ -9644,7 +9867,7 @@
         <v>7</v>
       </c>
       <c r="F7" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A7,Pendências!$B$2:$B$145,"Alta")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A7,Pendências!$B$2:$B$149,"Alta")</f>
         <v>2</v>
       </c>
     </row>
@@ -9653,15 +9876,15 @@
         <v>94</v>
       </c>
       <c r="B8" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A8,Pendências!$J$2:$J$145,"Vencida")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A8,Pendências!$J$2:$J$149,"Vencida")</f>
         <v>2</v>
       </c>
       <c r="C8" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A8,Pendências!$J$2:$J$145,"Sem data")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A8,Pendências!$J$2:$J$149,"Sem data")</f>
         <v>2</v>
       </c>
       <c r="D8" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A8,Pendências!$J$2:$J$145,"Vence em breve")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A8,Pendências!$J$2:$J$149,"Vence em breve")</f>
         <v>0</v>
       </c>
       <c r="E8" s="7" t="n">
@@ -9669,7 +9892,7 @@
         <v>4</v>
       </c>
       <c r="F8" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A8,Pendências!$B$2:$B$145,"Alta")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A8,Pendências!$B$2:$B$149,"Alta")</f>
         <v>1</v>
       </c>
     </row>
@@ -9678,15 +9901,15 @@
         <v>101</v>
       </c>
       <c r="B9" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A9,Pendências!$J$2:$J$145,"Vencida")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A9,Pendências!$J$2:$J$149,"Vencida")</f>
         <v>0</v>
       </c>
       <c r="C9" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A9,Pendências!$J$2:$J$145,"Sem data")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A9,Pendências!$J$2:$J$149,"Sem data")</f>
         <v>1</v>
       </c>
       <c r="D9" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A9,Pendências!$J$2:$J$145,"Vence em breve")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A9,Pendências!$J$2:$J$149,"Vence em breve")</f>
         <v>0</v>
       </c>
       <c r="E9" s="7" t="n">
@@ -9694,7 +9917,7 @@
         <v>1</v>
       </c>
       <c r="F9" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A9,Pendências!$B$2:$B$145,"Alta")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A9,Pendências!$B$2:$B$149,"Alta")</f>
         <v>0</v>
       </c>
     </row>
@@ -9703,15 +9926,15 @@
         <v>105</v>
       </c>
       <c r="B10" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A10,Pendências!$J$2:$J$145,"Vencida")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A10,Pendências!$J$2:$J$149,"Vencida")</f>
         <v>1</v>
       </c>
       <c r="C10" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A10,Pendências!$J$2:$J$145,"Sem data")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A10,Pendências!$J$2:$J$149,"Sem data")</f>
         <v>2</v>
       </c>
       <c r="D10" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A10,Pendências!$J$2:$J$145,"Vence em breve")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A10,Pendências!$J$2:$J$149,"Vence em breve")</f>
         <v>1</v>
       </c>
       <c r="E10" s="7" t="n">
@@ -9719,7 +9942,7 @@
         <v>4</v>
       </c>
       <c r="F10" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A10,Pendências!$B$2:$B$145,"Alta")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A10,Pendências!$B$2:$B$149,"Alta")</f>
         <v>1</v>
       </c>
     </row>
@@ -9728,15 +9951,15 @@
         <v>111</v>
       </c>
       <c r="B11" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A11,Pendências!$J$2:$J$145,"Vencida")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A11,Pendências!$J$2:$J$149,"Vencida")</f>
         <v>0</v>
       </c>
       <c r="C11" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A11,Pendências!$J$2:$J$145,"Sem data")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A11,Pendências!$J$2:$J$149,"Sem data")</f>
         <v>2</v>
       </c>
       <c r="D11" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A11,Pendências!$J$2:$J$145,"Vence em breve")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A11,Pendências!$J$2:$J$149,"Vence em breve")</f>
         <v>0</v>
       </c>
       <c r="E11" s="7" t="n">
@@ -9744,7 +9967,7 @@
         <v>2</v>
       </c>
       <c r="F11" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A11,Pendências!$B$2:$B$145,"Alta")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A11,Pendências!$B$2:$B$149,"Alta")</f>
         <v>0</v>
       </c>
     </row>
@@ -9753,15 +9976,15 @@
         <v>115</v>
       </c>
       <c r="B12" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A12,Pendências!$J$2:$J$145,"Vencida")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A12,Pendências!$J$2:$J$149,"Vencida")</f>
         <v>3</v>
       </c>
       <c r="C12" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A12,Pendências!$J$2:$J$145,"Sem data")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A12,Pendências!$J$2:$J$149,"Sem data")</f>
         <v>3</v>
       </c>
       <c r="D12" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A12,Pendências!$J$2:$J$145,"Vence em breve")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A12,Pendências!$J$2:$J$149,"Vence em breve")</f>
         <v>0</v>
       </c>
       <c r="E12" s="7" t="n">
@@ -9769,7 +9992,7 @@
         <v>6</v>
       </c>
       <c r="F12" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A12,Pendências!$B$2:$B$145,"Alta")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A12,Pendências!$B$2:$B$149,"Alta")</f>
         <v>1</v>
       </c>
     </row>
@@ -9778,15 +10001,15 @@
         <v>119</v>
       </c>
       <c r="B13" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A13,Pendências!$J$2:$J$145,"Vencida")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A13,Pendências!$J$2:$J$149,"Vencida")</f>
         <v>1</v>
       </c>
       <c r="C13" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A13,Pendências!$J$2:$J$145,"Sem data")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A13,Pendências!$J$2:$J$149,"Sem data")</f>
         <v>0</v>
       </c>
       <c r="D13" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A13,Pendências!$J$2:$J$145,"Vence em breve")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A13,Pendências!$J$2:$J$149,"Vence em breve")</f>
         <v>0</v>
       </c>
       <c r="E13" s="7" t="n">
@@ -9794,7 +10017,7 @@
         <v>1</v>
       </c>
       <c r="F13" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A13,Pendências!$B$2:$B$145,"Alta")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A13,Pendências!$B$2:$B$149,"Alta")</f>
         <v>1</v>
       </c>
     </row>
@@ -9803,15 +10026,15 @@
         <v>123</v>
       </c>
       <c r="B14" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A14,Pendências!$J$2:$J$145,"Vencida")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A14,Pendências!$J$2:$J$149,"Vencida")</f>
         <v>2</v>
       </c>
       <c r="C14" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A14,Pendências!$J$2:$J$145,"Sem data")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A14,Pendências!$J$2:$J$149,"Sem data")</f>
         <v>0</v>
       </c>
       <c r="D14" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A14,Pendências!$J$2:$J$145,"Vence em breve")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A14,Pendências!$J$2:$J$149,"Vence em breve")</f>
         <v>1</v>
       </c>
       <c r="E14" s="7" t="n">
@@ -9819,7 +10042,7 @@
         <v>3</v>
       </c>
       <c r="F14" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A14,Pendências!$B$2:$B$145,"Alta")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A14,Pendências!$B$2:$B$149,"Alta")</f>
         <v>1</v>
       </c>
     </row>
@@ -9828,15 +10051,15 @@
         <v>127</v>
       </c>
       <c r="B15" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A15,Pendências!$J$2:$J$145,"Vencida")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A15,Pendências!$J$2:$J$149,"Vencida")</f>
         <v>2</v>
       </c>
       <c r="C15" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A15,Pendências!$J$2:$J$145,"Sem data")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A15,Pendências!$J$2:$J$149,"Sem data")</f>
         <v>0</v>
       </c>
       <c r="D15" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A15,Pendências!$J$2:$J$145,"Vence em breve")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A15,Pendências!$J$2:$J$149,"Vence em breve")</f>
         <v>0</v>
       </c>
       <c r="E15" s="7" t="n">
@@ -9844,7 +10067,7 @@
         <v>2</v>
       </c>
       <c r="F15" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A15,Pendências!$B$2:$B$145,"Alta")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A15,Pendências!$B$2:$B$149,"Alta")</f>
         <v>2</v>
       </c>
     </row>
@@ -9853,15 +10076,15 @@
         <v>132</v>
       </c>
       <c r="B16" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A16,Pendências!$J$2:$J$145,"Vencida")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A16,Pendências!$J$2:$J$149,"Vencida")</f>
         <v>3</v>
       </c>
       <c r="C16" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A16,Pendências!$J$2:$J$145,"Sem data")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A16,Pendências!$J$2:$J$149,"Sem data")</f>
         <v>1</v>
       </c>
       <c r="D16" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A16,Pendências!$J$2:$J$145,"Vence em breve")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A16,Pendências!$J$2:$J$149,"Vence em breve")</f>
         <v>0</v>
       </c>
       <c r="E16" s="7" t="n">
@@ -9869,7 +10092,7 @@
         <v>4</v>
       </c>
       <c r="F16" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A16,Pendências!$B$2:$B$145,"Alta")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A16,Pendências!$B$2:$B$149,"Alta")</f>
         <v>2</v>
       </c>
     </row>
@@ -9878,15 +10101,15 @@
         <v>139</v>
       </c>
       <c r="B17" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A17,Pendências!$J$2:$J$145,"Vencida")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A17,Pendências!$J$2:$J$149,"Vencida")</f>
         <v>1</v>
       </c>
       <c r="C17" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A17,Pendências!$J$2:$J$145,"Sem data")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A17,Pendências!$J$2:$J$149,"Sem data")</f>
         <v>0</v>
       </c>
       <c r="D17" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A17,Pendências!$J$2:$J$145,"Vence em breve")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A17,Pendências!$J$2:$J$149,"Vence em breve")</f>
         <v>0</v>
       </c>
       <c r="E17" s="7" t="n">
@@ -9894,7 +10117,7 @@
         <v>1</v>
       </c>
       <c r="F17" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A17,Pendências!$B$2:$B$145,"Alta")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A17,Pendências!$B$2:$B$149,"Alta")</f>
         <v>1</v>
       </c>
     </row>
@@ -9903,15 +10126,15 @@
         <v>143</v>
       </c>
       <c r="B18" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A18,Pendências!$J$2:$J$145,"Vencida")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A18,Pendências!$J$2:$J$149,"Vencida")</f>
         <v>4</v>
       </c>
       <c r="C18" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A18,Pendências!$J$2:$J$145,"Sem data")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A18,Pendências!$J$2:$J$149,"Sem data")</f>
         <v>2</v>
       </c>
       <c r="D18" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A18,Pendências!$J$2:$J$145,"Vence em breve")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A18,Pendências!$J$2:$J$149,"Vence em breve")</f>
         <v>1</v>
       </c>
       <c r="E18" s="7" t="n">
@@ -9919,7 +10142,7 @@
         <v>7</v>
       </c>
       <c r="F18" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A18,Pendências!$B$2:$B$145,"Alta")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A18,Pendências!$B$2:$B$149,"Alta")</f>
         <v>2</v>
       </c>
     </row>
@@ -9928,15 +10151,15 @@
         <v>148</v>
       </c>
       <c r="B19" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A19,Pendências!$J$2:$J$145,"Vencida")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A19,Pendências!$J$2:$J$149,"Vencida")</f>
         <v>2</v>
       </c>
       <c r="C19" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A19,Pendências!$J$2:$J$145,"Sem data")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A19,Pendências!$J$2:$J$149,"Sem data")</f>
         <v>1</v>
       </c>
       <c r="D19" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A19,Pendências!$J$2:$J$145,"Vence em breve")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A19,Pendências!$J$2:$J$149,"Vence em breve")</f>
         <v>1</v>
       </c>
       <c r="E19" s="7" t="n">
@@ -9944,7 +10167,7 @@
         <v>4</v>
       </c>
       <c r="F19" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A19,Pendências!$B$2:$B$145,"Alta")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A19,Pendências!$B$2:$B$149,"Alta")</f>
         <v>1</v>
       </c>
     </row>
@@ -9953,15 +10176,15 @@
         <v>154</v>
       </c>
       <c r="B20" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A20,Pendências!$J$2:$J$145,"Vencida")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A20,Pendências!$J$2:$J$149,"Vencida")</f>
         <v>1</v>
       </c>
       <c r="C20" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A20,Pendências!$J$2:$J$145,"Sem data")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A20,Pendências!$J$2:$J$149,"Sem data")</f>
         <v>0</v>
       </c>
       <c r="D20" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A20,Pendências!$J$2:$J$145,"Vence em breve")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A20,Pendências!$J$2:$J$149,"Vence em breve")</f>
         <v>0</v>
       </c>
       <c r="E20" s="7" t="n">
@@ -9969,7 +10192,7 @@
         <v>1</v>
       </c>
       <c r="F20" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A20,Pendências!$B$2:$B$145,"Alta")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A20,Pendências!$B$2:$B$149,"Alta")</f>
         <v>1</v>
       </c>
     </row>
@@ -9978,15 +10201,15 @@
         <v>157</v>
       </c>
       <c r="B21" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A21,Pendências!$J$2:$J$145,"Vencida")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A21,Pendências!$J$2:$J$149,"Vencida")</f>
         <v>1</v>
       </c>
       <c r="C21" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A21,Pendências!$J$2:$J$145,"Sem data")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A21,Pendências!$J$2:$J$149,"Sem data")</f>
         <v>2</v>
       </c>
       <c r="D21" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A21,Pendências!$J$2:$J$145,"Vence em breve")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A21,Pendências!$J$2:$J$149,"Vence em breve")</f>
         <v>0</v>
       </c>
       <c r="E21" s="7" t="n">
@@ -9994,7 +10217,7 @@
         <v>3</v>
       </c>
       <c r="F21" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A21,Pendências!$B$2:$B$145,"Alta")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A21,Pendências!$B$2:$B$149,"Alta")</f>
         <v>0</v>
       </c>
     </row>
@@ -10003,15 +10226,15 @@
         <v>163</v>
       </c>
       <c r="B22" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A22,Pendências!$J$2:$J$145,"Vencida")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A22,Pendências!$J$2:$J$149,"Vencida")</f>
         <v>2</v>
       </c>
       <c r="C22" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A22,Pendências!$J$2:$J$145,"Sem data")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A22,Pendências!$J$2:$J$149,"Sem data")</f>
         <v>1</v>
       </c>
       <c r="D22" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A22,Pendências!$J$2:$J$145,"Vence em breve")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A22,Pendências!$J$2:$J$149,"Vence em breve")</f>
         <v>0</v>
       </c>
       <c r="E22" s="7" t="n">
@@ -10019,7 +10242,7 @@
         <v>3</v>
       </c>
       <c r="F22" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A22,Pendências!$B$2:$B$145,"Alta")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A22,Pendências!$B$2:$B$149,"Alta")</f>
         <v>2</v>
       </c>
     </row>
@@ -10028,15 +10251,15 @@
         <v>166</v>
       </c>
       <c r="B23" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A23,Pendências!$J$2:$J$145,"Vencida")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A23,Pendências!$J$2:$J$149,"Vencida")</f>
         <v>1</v>
       </c>
       <c r="C23" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A23,Pendências!$J$2:$J$145,"Sem data")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A23,Pendências!$J$2:$J$149,"Sem data")</f>
         <v>1</v>
       </c>
       <c r="D23" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A23,Pendências!$J$2:$J$145,"Vence em breve")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A23,Pendências!$J$2:$J$149,"Vence em breve")</f>
         <v>0</v>
       </c>
       <c r="E23" s="7" t="n">
@@ -10044,7 +10267,7 @@
         <v>2</v>
       </c>
       <c r="F23" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A23,Pendências!$B$2:$B$145,"Alta")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A23,Pendências!$B$2:$B$149,"Alta")</f>
         <v>1</v>
       </c>
     </row>
@@ -10053,15 +10276,15 @@
         <v>170</v>
       </c>
       <c r="B24" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A24,Pendências!$J$2:$J$145,"Vencida")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A24,Pendências!$J$2:$J$149,"Vencida")</f>
         <v>1</v>
       </c>
       <c r="C24" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A24,Pendências!$J$2:$J$145,"Sem data")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A24,Pendências!$J$2:$J$149,"Sem data")</f>
         <v>0</v>
       </c>
       <c r="D24" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A24,Pendências!$J$2:$J$145,"Vence em breve")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A24,Pendências!$J$2:$J$149,"Vence em breve")</f>
         <v>0</v>
       </c>
       <c r="E24" s="7" t="n">
@@ -10069,7 +10292,7 @@
         <v>1</v>
       </c>
       <c r="F24" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A24,Pendências!$B$2:$B$145,"Alta")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A24,Pendências!$B$2:$B$149,"Alta")</f>
         <v>1</v>
       </c>
     </row>
@@ -10078,15 +10301,15 @@
         <v>174</v>
       </c>
       <c r="B25" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A25,Pendências!$J$2:$J$145,"Vencida")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A25,Pendências!$J$2:$J$149,"Vencida")</f>
         <v>1</v>
       </c>
       <c r="C25" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A25,Pendências!$J$2:$J$145,"Sem data")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A25,Pendências!$J$2:$J$149,"Sem data")</f>
         <v>1</v>
       </c>
       <c r="D25" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A25,Pendências!$J$2:$J$145,"Vence em breve")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A25,Pendências!$J$2:$J$149,"Vence em breve")</f>
         <v>0</v>
       </c>
       <c r="E25" s="7" t="n">
@@ -10094,7 +10317,7 @@
         <v>2</v>
       </c>
       <c r="F25" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A25,Pendências!$B$2:$B$145,"Alta")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A25,Pendências!$B$2:$B$149,"Alta")</f>
         <v>1</v>
       </c>
     </row>
@@ -10103,15 +10326,15 @@
         <v>178</v>
       </c>
       <c r="B26" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A26,Pendências!$J$2:$J$145,"Vencida")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A26,Pendências!$J$2:$J$149,"Vencida")</f>
         <v>2</v>
       </c>
       <c r="C26" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A26,Pendências!$J$2:$J$145,"Sem data")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A26,Pendências!$J$2:$J$149,"Sem data")</f>
         <v>0</v>
       </c>
       <c r="D26" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A26,Pendências!$J$2:$J$145,"Vence em breve")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A26,Pendências!$J$2:$J$149,"Vence em breve")</f>
         <v>0</v>
       </c>
       <c r="E26" s="7" t="n">
@@ -10119,7 +10342,7 @@
         <v>2</v>
       </c>
       <c r="F26" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A26,Pendências!$B$2:$B$145,"Alta")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A26,Pendências!$B$2:$B$149,"Alta")</f>
         <v>2</v>
       </c>
     </row>
@@ -10128,15 +10351,15 @@
         <v>183</v>
       </c>
       <c r="B27" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A27,Pendências!$J$2:$J$145,"Vencida")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A27,Pendências!$J$2:$J$149,"Vencida")</f>
         <v>2</v>
       </c>
       <c r="C27" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A27,Pendências!$J$2:$J$145,"Sem data")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A27,Pendências!$J$2:$J$149,"Sem data")</f>
         <v>0</v>
       </c>
       <c r="D27" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A27,Pendências!$J$2:$J$145,"Vence em breve")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A27,Pendências!$J$2:$J$149,"Vence em breve")</f>
         <v>0</v>
       </c>
       <c r="E27" s="7" t="n">
@@ -10144,7 +10367,7 @@
         <v>2</v>
       </c>
       <c r="F27" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A27,Pendências!$B$2:$B$145,"Alta")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A27,Pendências!$B$2:$B$149,"Alta")</f>
         <v>2</v>
       </c>
     </row>
@@ -10153,15 +10376,15 @@
         <v>188</v>
       </c>
       <c r="B28" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A28,Pendências!$J$2:$J$145,"Vencida")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A28,Pendências!$J$2:$J$149,"Vencida")</f>
         <v>3</v>
       </c>
       <c r="C28" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A28,Pendências!$J$2:$J$145,"Sem data")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A28,Pendências!$J$2:$J$149,"Sem data")</f>
         <v>0</v>
       </c>
       <c r="D28" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A28,Pendências!$J$2:$J$145,"Vence em breve")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A28,Pendências!$J$2:$J$149,"Vence em breve")</f>
         <v>0</v>
       </c>
       <c r="E28" s="7" t="n">
@@ -10169,7 +10392,7 @@
         <v>3</v>
       </c>
       <c r="F28" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A28,Pendências!$B$2:$B$145,"Alta")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A28,Pendências!$B$2:$B$149,"Alta")</f>
         <v>2</v>
       </c>
     </row>
@@ -10178,15 +10401,15 @@
         <v>193</v>
       </c>
       <c r="B29" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A29,Pendências!$J$2:$J$145,"Vencida")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A29,Pendências!$J$2:$J$149,"Vencida")</f>
         <v>2</v>
       </c>
       <c r="C29" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A29,Pendências!$J$2:$J$145,"Sem data")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A29,Pendências!$J$2:$J$149,"Sem data")</f>
         <v>0</v>
       </c>
       <c r="D29" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A29,Pendências!$J$2:$J$145,"Vence em breve")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A29,Pendências!$J$2:$J$149,"Vence em breve")</f>
         <v>0</v>
       </c>
       <c r="E29" s="7" t="n">
@@ -10194,7 +10417,7 @@
         <v>2</v>
       </c>
       <c r="F29" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A29,Pendências!$B$2:$B$145,"Alta")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A29,Pendências!$B$2:$B$149,"Alta")</f>
         <v>1</v>
       </c>
     </row>
@@ -10203,15 +10426,15 @@
         <v>197</v>
       </c>
       <c r="B30" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A30,Pendências!$J$2:$J$145,"Vencida")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A30,Pendências!$J$2:$J$149,"Vencida")</f>
         <v>5</v>
       </c>
       <c r="C30" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A30,Pendências!$J$2:$J$145,"Sem data")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A30,Pendências!$J$2:$J$149,"Sem data")</f>
         <v>0</v>
       </c>
       <c r="D30" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A30,Pendências!$J$2:$J$145,"Vence em breve")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A30,Pendências!$J$2:$J$149,"Vence em breve")</f>
         <v>0</v>
       </c>
       <c r="E30" s="7" t="n">
@@ -10219,7 +10442,7 @@
         <v>5</v>
       </c>
       <c r="F30" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A30,Pendências!$B$2:$B$145,"Alta")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A30,Pendências!$B$2:$B$149,"Alta")</f>
         <v>3</v>
       </c>
     </row>
@@ -10228,15 +10451,15 @@
         <v>206</v>
       </c>
       <c r="B31" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A31,Pendências!$J$2:$J$145,"Vencida")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A31,Pendências!$J$2:$J$149,"Vencida")</f>
         <v>0</v>
       </c>
       <c r="C31" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A31,Pendências!$J$2:$J$145,"Sem data")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A31,Pendências!$J$2:$J$149,"Sem data")</f>
         <v>1</v>
       </c>
       <c r="D31" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A31,Pendências!$J$2:$J$145,"Vence em breve")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A31,Pendências!$J$2:$J$149,"Vence em breve")</f>
         <v>0</v>
       </c>
       <c r="E31" s="7" t="n">
@@ -10244,7 +10467,7 @@
         <v>1</v>
       </c>
       <c r="F31" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A31,Pendências!$B$2:$B$145,"Alta")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A31,Pendências!$B$2:$B$149,"Alta")</f>
         <v>0</v>
       </c>
     </row>
@@ -10253,15 +10476,15 @@
         <v>210</v>
       </c>
       <c r="B32" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A32,Pendências!$J$2:$J$145,"Vencida")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A32,Pendências!$J$2:$J$149,"Vencida")</f>
         <v>3</v>
       </c>
       <c r="C32" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A32,Pendências!$J$2:$J$145,"Sem data")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A32,Pendências!$J$2:$J$149,"Sem data")</f>
         <v>0</v>
       </c>
       <c r="D32" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A32,Pendências!$J$2:$J$145,"Vence em breve")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A32,Pendências!$J$2:$J$149,"Vence em breve")</f>
         <v>0</v>
       </c>
       <c r="E32" s="7" t="n">
@@ -10269,7 +10492,7 @@
         <v>3</v>
       </c>
       <c r="F32" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A32,Pendências!$B$2:$B$145,"Alta")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A32,Pendências!$B$2:$B$149,"Alta")</f>
         <v>2</v>
       </c>
     </row>
@@ -10278,15 +10501,15 @@
         <v>215</v>
       </c>
       <c r="B33" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A33,Pendências!$J$2:$J$145,"Vencida")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A33,Pendências!$J$2:$J$149,"Vencida")</f>
         <v>3</v>
       </c>
       <c r="C33" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A33,Pendências!$J$2:$J$145,"Sem data")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A33,Pendências!$J$2:$J$149,"Sem data")</f>
         <v>1</v>
       </c>
       <c r="D33" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A33,Pendências!$J$2:$J$145,"Vence em breve")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A33,Pendências!$J$2:$J$149,"Vence em breve")</f>
         <v>0</v>
       </c>
       <c r="E33" s="7" t="n">
@@ -10294,7 +10517,7 @@
         <v>4</v>
       </c>
       <c r="F33" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A33,Pendências!$B$2:$B$145,"Alta")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A33,Pendências!$B$2:$B$149,"Alta")</f>
         <v>2</v>
       </c>
     </row>
@@ -10303,15 +10526,15 @@
         <v>222</v>
       </c>
       <c r="B34" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A34,Pendências!$J$2:$J$145,"Vencida")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A34,Pendências!$J$2:$J$149,"Vencida")</f>
         <v>1</v>
       </c>
       <c r="C34" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A34,Pendências!$J$2:$J$145,"Sem data")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A34,Pendências!$J$2:$J$149,"Sem data")</f>
         <v>1</v>
       </c>
       <c r="D34" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A34,Pendências!$J$2:$J$145,"Vence em breve")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A34,Pendências!$J$2:$J$149,"Vence em breve")</f>
         <v>1</v>
       </c>
       <c r="E34" s="7" t="n">
@@ -10319,7 +10542,7 @@
         <v>3</v>
       </c>
       <c r="F34" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A34,Pendências!$B$2:$B$145,"Alta")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A34,Pendências!$B$2:$B$149,"Alta")</f>
         <v>2</v>
       </c>
     </row>
@@ -10328,15 +10551,15 @@
         <v>227</v>
       </c>
       <c r="B35" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A35,Pendências!$J$2:$J$145,"Vencida")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A35,Pendências!$J$2:$J$149,"Vencida")</f>
         <v>1</v>
       </c>
       <c r="C35" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A35,Pendências!$J$2:$J$145,"Sem data")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A35,Pendências!$J$2:$J$149,"Sem data")</f>
         <v>0</v>
       </c>
       <c r="D35" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A35,Pendências!$J$2:$J$145,"Vence em breve")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A35,Pendências!$J$2:$J$149,"Vence em breve")</f>
         <v>1</v>
       </c>
       <c r="E35" s="7" t="n">
@@ -10344,7 +10567,7 @@
         <v>2</v>
       </c>
       <c r="F35" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A35,Pendências!$B$2:$B$145,"Alta")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A35,Pendências!$B$2:$B$149,"Alta")</f>
         <v>1</v>
       </c>
     </row>
@@ -10353,15 +10576,15 @@
         <v>233</v>
       </c>
       <c r="B36" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A36,Pendências!$J$2:$J$145,"Vencida")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A36,Pendências!$J$2:$J$149,"Vencida")</f>
         <v>4</v>
       </c>
       <c r="C36" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A36,Pendências!$J$2:$J$145,"Sem data")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A36,Pendências!$J$2:$J$149,"Sem data")</f>
         <v>0</v>
       </c>
       <c r="D36" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A36,Pendências!$J$2:$J$145,"Vence em breve")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A36,Pendências!$J$2:$J$149,"Vence em breve")</f>
         <v>0</v>
       </c>
       <c r="E36" s="7" t="n">
@@ -10369,7 +10592,7 @@
         <v>4</v>
       </c>
       <c r="F36" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A36,Pendências!$B$2:$B$145,"Alta")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A36,Pendências!$B$2:$B$149,"Alta")</f>
         <v>3</v>
       </c>
     </row>
@@ -10378,15 +10601,15 @@
         <v>239</v>
       </c>
       <c r="B37" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A37,Pendências!$J$2:$J$145,"Vencida")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A37,Pendências!$J$2:$J$149,"Vencida")</f>
         <v>1</v>
       </c>
       <c r="C37" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A37,Pendências!$J$2:$J$145,"Sem data")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A37,Pendências!$J$2:$J$149,"Sem data")</f>
         <v>0</v>
       </c>
       <c r="D37" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A37,Pendências!$J$2:$J$145,"Vence em breve")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A37,Pendências!$J$2:$J$149,"Vence em breve")</f>
         <v>0</v>
       </c>
       <c r="E37" s="7" t="n">
@@ -10394,7 +10617,7 @@
         <v>1</v>
       </c>
       <c r="F37" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A37,Pendências!$B$2:$B$145,"Alta")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A37,Pendências!$B$2:$B$149,"Alta")</f>
         <v>1</v>
       </c>
     </row>
@@ -10403,15 +10626,15 @@
         <v>242</v>
       </c>
       <c r="B38" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A38,Pendências!$J$2:$J$145,"Vencida")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A38,Pendências!$J$2:$J$149,"Vencida")</f>
         <v>2</v>
       </c>
       <c r="C38" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A38,Pendências!$J$2:$J$145,"Sem data")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A38,Pendências!$J$2:$J$149,"Sem data")</f>
         <v>0</v>
       </c>
       <c r="D38" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A38,Pendências!$J$2:$J$145,"Vence em breve")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A38,Pendências!$J$2:$J$149,"Vence em breve")</f>
         <v>1</v>
       </c>
       <c r="E38" s="7" t="n">
@@ -10419,7 +10642,7 @@
         <v>3</v>
       </c>
       <c r="F38" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A38,Pendências!$B$2:$B$145,"Alta")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A38,Pendências!$B$2:$B$149,"Alta")</f>
         <v>3</v>
       </c>
     </row>
@@ -10428,15 +10651,15 @@
         <v>247</v>
       </c>
       <c r="B39" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A39,Pendências!$J$2:$J$145,"Vencida")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A39,Pendências!$J$2:$J$149,"Vencida")</f>
         <v>2</v>
       </c>
       <c r="C39" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A39,Pendências!$J$2:$J$145,"Sem data")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A39,Pendências!$J$2:$J$149,"Sem data")</f>
         <v>0</v>
       </c>
       <c r="D39" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A39,Pendências!$J$2:$J$145,"Vence em breve")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A39,Pendências!$J$2:$J$149,"Vence em breve")</f>
         <v>0</v>
       </c>
       <c r="E39" s="7" t="n">
@@ -10444,7 +10667,7 @@
         <v>2</v>
       </c>
       <c r="F39" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A39,Pendências!$B$2:$B$145,"Alta")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A39,Pendências!$B$2:$B$149,"Alta")</f>
         <v>2</v>
       </c>
     </row>
@@ -10453,15 +10676,15 @@
         <v>252</v>
       </c>
       <c r="B40" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A40,Pendências!$J$2:$J$145,"Vencida")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A40,Pendências!$J$2:$J$149,"Vencida")</f>
         <v>3</v>
       </c>
       <c r="C40" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A40,Pendências!$J$2:$J$145,"Sem data")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A40,Pendências!$J$2:$J$149,"Sem data")</f>
         <v>0</v>
       </c>
       <c r="D40" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A40,Pendências!$J$2:$J$145,"Vence em breve")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A40,Pendências!$J$2:$J$149,"Vence em breve")</f>
         <v>0</v>
       </c>
       <c r="E40" s="7" t="n">
@@ -10469,7 +10692,7 @@
         <v>3</v>
       </c>
       <c r="F40" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A40,Pendências!$B$2:$B$145,"Alta")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A40,Pendências!$B$2:$B$149,"Alta")</f>
         <v>3</v>
       </c>
     </row>
@@ -10478,15 +10701,15 @@
         <v>258</v>
       </c>
       <c r="B41" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A41,Pendências!$J$2:$J$145,"Vencida")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A41,Pendências!$J$2:$J$149,"Vencida")</f>
         <v>2</v>
       </c>
       <c r="C41" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A41,Pendências!$J$2:$J$145,"Sem data")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A41,Pendências!$J$2:$J$149,"Sem data")</f>
         <v>0</v>
       </c>
       <c r="D41" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A41,Pendências!$J$2:$J$145,"Vence em breve")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A41,Pendências!$J$2:$J$149,"Vence em breve")</f>
         <v>0</v>
       </c>
       <c r="E41" s="7" t="n">
@@ -10494,7 +10717,7 @@
         <v>2</v>
       </c>
       <c r="F41" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A41,Pendências!$B$2:$B$145,"Alta")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A41,Pendências!$B$2:$B$149,"Alta")</f>
         <v>2</v>
       </c>
     </row>
@@ -10503,24 +10726,24 @@
         <v>263</v>
       </c>
       <c r="B42" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A42,Pendências!$J$2:$J$145,"Vencida")</f>
-        <v>3</v>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A42,Pendências!$J$2:$J$149,"Vencida")</f>
+        <v>2</v>
       </c>
       <c r="C42" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A42,Pendências!$J$2:$J$145,"Sem data")</f>
-        <v>0</v>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A42,Pendências!$J$2:$J$149,"Sem data")</f>
+        <v>1</v>
       </c>
       <c r="D42" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A42,Pendências!$J$2:$J$145,"Vence em breve")</f>
-        <v>0</v>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A42,Pendências!$J$2:$J$149,"Vence em breve")</f>
+        <v>1</v>
       </c>
       <c r="E42" s="7" t="n">
         <f aca="false">SUM(B42:D42)</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="F42" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A42,Pendências!$B$2:$B$145,"Alta")</f>
-        <v>3</v>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A42,Pendências!$B$2:$B$149,"Alta")</f>
+        <v>2</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -10528,15 +10751,15 @@
         <v>270</v>
       </c>
       <c r="B43" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A43,Pendências!$J$2:$J$145,"Vencida")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A43,Pendências!$J$2:$J$149,"Vencida")</f>
         <v>3</v>
       </c>
       <c r="C43" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A43,Pendências!$J$2:$J$145,"Sem data")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A43,Pendências!$J$2:$J$149,"Sem data")</f>
         <v>0</v>
       </c>
       <c r="D43" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A43,Pendências!$J$2:$J$145,"Vence em breve")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A43,Pendências!$J$2:$J$149,"Vence em breve")</f>
         <v>0</v>
       </c>
       <c r="E43" s="7" t="n">
@@ -10544,24 +10767,24 @@
         <v>3</v>
       </c>
       <c r="F43" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A43,Pendências!$B$2:$B$145,"Alta")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A43,Pendências!$B$2:$B$149,"Alta")</f>
         <v>3</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="6" t="s">
-        <v>274</v>
+        <v>277</v>
       </c>
       <c r="B44" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A44,Pendências!$J$2:$J$145,"Vencida")</f>
-        <v>1</v>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A44,Pendências!$J$2:$J$149,"Vencida")</f>
+        <v>3</v>
       </c>
       <c r="C44" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A44,Pendências!$J$2:$J$145,"Sem data")</f>
-        <v>2</v>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A44,Pendências!$J$2:$J$149,"Sem data")</f>
+        <v>0</v>
       </c>
       <c r="D44" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A44,Pendências!$J$2:$J$145,"Vence em breve")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A44,Pendências!$J$2:$J$149,"Vence em breve")</f>
         <v>0</v>
       </c>
       <c r="E44" s="7" t="n">
@@ -10569,24 +10792,24 @@
         <v>3</v>
       </c>
       <c r="F44" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A44,Pendências!$B$2:$B$145,"Alta")</f>
-        <v>1</v>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A44,Pendências!$B$2:$B$149,"Alta")</f>
+        <v>3</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="6" t="s">
-        <v>278</v>
+        <v>281</v>
       </c>
       <c r="B45" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A45,Pendências!$J$2:$J$145,"Vencida")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A45,Pendências!$J$2:$J$149,"Vencida")</f>
+        <v>1</v>
+      </c>
+      <c r="C45" s="6" t="n">
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A45,Pendências!$J$2:$J$149,"Sem data")</f>
         <v>2</v>
       </c>
-      <c r="C45" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A45,Pendências!$J$2:$J$145,"Sem data")</f>
-        <v>1</v>
-      </c>
       <c r="D45" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A45,Pendências!$J$2:$J$145,"Vence em breve")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A45,Pendências!$J$2:$J$149,"Vence em breve")</f>
         <v>0</v>
       </c>
       <c r="E45" s="7" t="n">
@@ -10594,32 +10817,32 @@
         <v>3</v>
       </c>
       <c r="F45" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A45,Pendências!$B$2:$B$145,"Alta")</f>
-        <v>2</v>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A45,Pendências!$B$2:$B$149,"Alta")</f>
+        <v>1</v>
       </c>
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="6" t="s">
-        <v>282</v>
+        <v>285</v>
       </c>
       <c r="B46" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A46,Pendências!$J$2:$J$145,"Vencida")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A46,Pendências!$J$2:$J$149,"Vencida")</f>
         <v>2</v>
       </c>
       <c r="C46" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A46,Pendências!$J$2:$J$145,"Sem data")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A46,Pendências!$J$2:$J$149,"Sem data")</f>
+        <v>1</v>
+      </c>
+      <c r="D46" s="6" t="n">
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A46,Pendências!$J$2:$J$149,"Vence em breve")</f>
         <v>0</v>
-      </c>
-      <c r="D46" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A46,Pendências!$J$2:$J$145,"Vence em breve")</f>
-        <v>1</v>
       </c>
       <c r="E46" s="7" t="n">
         <f aca="false">SUM(B46:D46)</f>
         <v>3</v>
       </c>
       <c r="F46" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A46,Pendências!$B$2:$B$145,"Alta")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A46,Pendências!$B$2:$B$149,"Alta")</f>
         <v>2</v>
       </c>
     </row>
@@ -10628,103 +10851,128 @@
         <v>289</v>
       </c>
       <c r="B47" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A47,Pendências!$J$2:$J$145,"Vencida")</f>
-        <v>4</v>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A47,Pendências!$J$2:$J$149,"Vencida")</f>
+        <v>2</v>
       </c>
       <c r="C47" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A47,Pendências!$J$2:$J$145,"Sem data")</f>
-        <v>1</v>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A47,Pendências!$J$2:$J$149,"Sem data")</f>
+        <v>0</v>
       </c>
       <c r="D47" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A47,Pendências!$J$2:$J$145,"Vence em breve")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A47,Pendências!$J$2:$J$149,"Vence em breve")</f>
         <v>1</v>
       </c>
       <c r="E47" s="7" t="n">
         <f aca="false">SUM(B47:D47)</f>
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F47" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A47,Pendências!$B$2:$B$145,"Alta")</f>
-        <v>4</v>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A47,Pendências!$B$2:$B$149,"Alta")</f>
+        <v>2</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="6" t="s">
-        <v>295</v>
+        <v>296</v>
       </c>
       <c r="B48" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A48,Pendências!$J$2:$J$145,"Vencida")</f>
-        <v>3</v>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A48,Pendências!$J$2:$J$149,"Vencida")</f>
+        <v>4</v>
       </c>
       <c r="C48" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A48,Pendências!$J$2:$J$145,"Sem data")</f>
-        <v>4</v>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A48,Pendências!$J$2:$J$149,"Sem data")</f>
+        <v>1</v>
       </c>
       <c r="D48" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A48,Pendências!$J$2:$J$145,"Vence em breve")</f>
-        <v>0</v>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A48,Pendências!$J$2:$J$149,"Vence em breve")</f>
+        <v>1</v>
       </c>
       <c r="E48" s="7" t="n">
         <f aca="false">SUM(B48:D48)</f>
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F48" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A48,Pendências!$B$2:$B$145,"Alta")</f>
-        <v>1</v>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A48,Pendências!$B$2:$B$149,"Alta")</f>
+        <v>4</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="6" t="s">
-        <v>300</v>
+        <v>302</v>
       </c>
       <c r="B49" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A49,Pendências!$J$2:$J$145,"Vencida")</f>
-        <v>2</v>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A49,Pendências!$J$2:$J$149,"Vencida")</f>
+        <v>3</v>
       </c>
       <c r="C49" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A49,Pendências!$J$2:$J$145,"Sem data")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A49,Pendências!$J$2:$J$149,"Sem data")</f>
+        <v>4</v>
+      </c>
+      <c r="D49" s="6" t="n">
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A49,Pendências!$J$2:$J$149,"Vence em breve")</f>
         <v>0</v>
-      </c>
-      <c r="D49" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A49,Pendências!$J$2:$J$145,"Vence em breve")</f>
-        <v>1</v>
       </c>
       <c r="E49" s="7" t="n">
         <f aca="false">SUM(B49:D49)</f>
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="F49" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A49,Pendências!$B$2:$B$145,"Alta")</f>
-        <v>2</v>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A49,Pendências!$B$2:$B$149,"Alta")</f>
+        <v>1</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="6" t="s">
-        <v>303</v>
+        <v>307</v>
       </c>
       <c r="B50" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A50,Pendências!$J$2:$J$145,"Vencida")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A50,Pendências!$J$2:$J$149,"Vencida")</f>
         <v>2</v>
       </c>
       <c r="C50" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A50,Pendências!$J$2:$J$145,"Sem data")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A50,Pendências!$J$2:$J$149,"Sem data")</f>
+        <v>0</v>
+      </c>
+      <c r="D50" s="6" t="n">
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A50,Pendências!$J$2:$J$149,"Vence em breve")</f>
         <v>1</v>
-      </c>
-      <c r="D50" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A50,Pendências!$J$2:$J$145,"Vence em breve")</f>
-        <v>0</v>
       </c>
       <c r="E50" s="7" t="n">
         <f aca="false">SUM(B50:D50)</f>
         <v>3</v>
       </c>
       <c r="F50" s="6" t="n">
-        <f aca="false">COUNTIFS(Pendências!$C$2:$C$145,$A50,Pendências!$B$2:$B$145,"Alta")</f>
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A50,Pendências!$B$2:$B$149,"Alta")</f>
         <v>2</v>
       </c>
     </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="6" t="s">
+        <v>310</v>
+      </c>
+      <c r="B51" s="6" t="n">
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A51,Pendências!$J$2:$J$149,"Vencida")</f>
+        <v>2</v>
+      </c>
+      <c r="C51" s="6" t="n">
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A51,Pendências!$J$2:$J$149,"Sem data")</f>
+        <v>1</v>
+      </c>
+      <c r="D51" s="6" t="n">
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A51,Pendências!$J$2:$J$149,"Vence em breve")</f>
+        <v>0</v>
+      </c>
+      <c r="E51" s="7" t="n">
+        <f aca="false">SUM(B51:D51)</f>
+        <v>3</v>
+      </c>
+      <c r="F51" s="6" t="n">
+        <f aca="false">COUNTIFS(Pendências!$C$2:$C$149,$A51,Pendências!$B$2:$B$149,"Alta")</f>
+        <v>2</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:F50"/>
+  <autoFilter ref="A1:F51"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -10769,167 +11017,167 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="17" t="s">
-        <v>309</v>
+        <v>316</v>
       </c>
       <c r="B2" s="17" t="s">
-        <v>310</v>
+        <v>317</v>
       </c>
       <c r="C2" s="17" t="s">
-        <v>311</v>
+        <v>318</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="17" t="s">
-        <v>312</v>
+        <v>319</v>
       </c>
       <c r="B3" s="17" t="s">
-        <v>313</v>
+        <v>320</v>
       </c>
       <c r="C3" s="17" t="s">
-        <v>314</v>
+        <v>321</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="17" t="s">
-        <v>315</v>
+        <v>322</v>
       </c>
       <c r="B4" s="17" t="s">
-        <v>316</v>
+        <v>323</v>
       </c>
       <c r="C4" s="17" t="s">
-        <v>317</v>
+        <v>324</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="17" t="s">
-        <v>318</v>
+        <v>325</v>
       </c>
       <c r="B5" s="17" t="s">
-        <v>319</v>
+        <v>326</v>
       </c>
       <c r="C5" s="17" t="s">
-        <v>320</v>
+        <v>327</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="17" t="s">
-        <v>321</v>
+        <v>328</v>
       </c>
       <c r="B6" s="17" t="s">
-        <v>322</v>
+        <v>329</v>
       </c>
       <c r="C6" s="17" t="s">
-        <v>323</v>
+        <v>330</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="17" t="s">
-        <v>324</v>
+        <v>331</v>
       </c>
       <c r="B7" s="17" t="s">
-        <v>325</v>
+        <v>332</v>
       </c>
       <c r="C7" s="17" t="s">
-        <v>326</v>
+        <v>333</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="17" t="s">
-        <v>327</v>
+        <v>334</v>
       </c>
       <c r="B8" s="17" t="s">
-        <v>328</v>
+        <v>335</v>
       </c>
       <c r="C8" s="17" t="s">
-        <v>329</v>
+        <v>336</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="17" t="s">
-        <v>330</v>
+        <v>337</v>
       </c>
       <c r="B9" s="17" t="s">
-        <v>322</v>
+        <v>329</v>
       </c>
       <c r="C9" s="17" t="s">
-        <v>331</v>
+        <v>338</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="17" t="s">
-        <v>332</v>
+        <v>339</v>
       </c>
       <c r="B10" s="17" t="s">
-        <v>333</v>
+        <v>340</v>
       </c>
       <c r="C10" s="17" t="s">
-        <v>334</v>
+        <v>341</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="17" t="s">
-        <v>335</v>
+        <v>342</v>
       </c>
       <c r="B11" s="17" t="s">
-        <v>336</v>
+        <v>343</v>
       </c>
       <c r="C11" s="17" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="17" t="s">
-        <v>338</v>
+        <v>345</v>
       </c>
       <c r="B12" s="17" t="s">
-        <v>339</v>
+        <v>346</v>
       </c>
       <c r="C12" s="17" t="s">
-        <v>340</v>
+        <v>347</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="17" t="s">
-        <v>341</v>
+        <v>348</v>
       </c>
       <c r="B13" s="17" t="s">
-        <v>342</v>
+        <v>349</v>
       </c>
       <c r="C13" s="17" t="s">
-        <v>343</v>
+        <v>350</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="17" t="s">
-        <v>344</v>
+        <v>351</v>
       </c>
       <c r="B14" s="17" t="s">
         <v>107</v>
       </c>
       <c r="C14" s="17" t="s">
-        <v>345</v>
+        <v>352</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="17" t="s">
-        <v>346</v>
+        <v>353</v>
       </c>
       <c r="B15" s="17" t="s">
-        <v>322</v>
+        <v>329</v>
       </c>
       <c r="C15" s="17" t="s">
-        <v>347</v>
+        <v>354</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="17" t="s">
-        <v>348</v>
+        <v>355</v>
       </c>
       <c r="B16" s="17" t="s">
-        <v>322</v>
+        <v>329</v>
       </c>
       <c r="C16" s="17" t="s">
-        <v>349</v>
+        <v>356</v>
       </c>
     </row>
   </sheetData>

</xml_diff>